<commit_message>
Off-prem MPO: 9/15 refresh of all four exports, Promos_Report_22, Keystone sync
Constellation 889 -> 971 placements this fall; Keystone 123 -> 146
buying accounts (Klejdi Lamo is the fifth rep at 40%); Fever Tree
87 -> 97 new placements (Chris Payton 0 -> 9); Wine & Spirits
186 -> 213 (Alex Rodriguez is the 18th rep at goal); cooler doors
31 -> 33 stickers with Mike Ast the fourth rep at goal. Same Keystone
export onto keystone-ice/actuals.csv and incentive-tracking rebuilt
(Klejdi qualifies, $470 -> $530). Hub cache tag bumped so it picks up
the new program_data.js.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019JKq7aCtXGsNtv2Y6TRt9r
</commit_message>
<xml_diff>
--- a/MPOs/off-prem/pos_cooler_door_promos.xlsx
+++ b/MPOs/off-prem/pos_cooler_door_promos.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q40"/>
+  <dimension ref="A1:Q45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21.7109375" customWidth="1" style="6" min="1" max="1"/>
@@ -591,7 +591,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>09/14/2026 09:50 AM</t>
+          <t>09/15/2026 12:07 PM</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -601,7 +601,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Shane Barreca</t>
+          <t>Mike Ast</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -625,26 +625,26 @@
         </is>
       </c>
       <c r="H2" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>SHOP RITE LIQ (A)HILLSDAL</t>
+          <t>WALDWICK WINE/SPIRITS</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>73008</t>
+          <t>88005</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>371 BROADWAY</t>
+          <t>23 WYCKOFF AVE</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>HILLSDALE</t>
+          <t>WALDWICK</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -659,12 +659,12 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>TWISTED TEA ORIGINAL</t>
+          <t>POP SIPS GINGER LIME</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>PASSION TREE</t>
         </is>
       </c>
       <c r="Q2" s="3" t="inlineStr">
@@ -676,17 +676,17 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>09/14/2026 07:38 AM</t>
+          <t>09/15/2026 12:07 PM</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Shane Barreca</t>
+          <t>Mike Ast</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -714,22 +714,22 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>WINEMART DISCOUNT</t>
+          <t>WALDWICK WINE/SPIRITS</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>74005</t>
+          <t>88005</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>700 BROADWAY SUITE 42</t>
+          <t>23 WYCKOFF AVE</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>WESTWOOD</t>
+          <t>WALDWICK</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -744,12 +744,12 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>NIGHT SHIFT X CAPE MAY BREWBERRY</t>
+          <t>POP SIPS RASPBERRY ROSE</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>NIGHT SHIFT BREWING</t>
+          <t>PASSION TREE</t>
         </is>
       </c>
       <c r="Q3" s="3" t="inlineStr">
@@ -761,17 +761,17 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>09/14/2026 07:36 AM</t>
+          <t>09/15/2026 12:07 PM</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Shane Barreca</t>
+          <t>Mike Ast</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -799,22 +799,22 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>WESTWOOD WINE AND LIQUORS</t>
+          <t>WALDWICK WINE/SPIRITS</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>74009</t>
+          <t>88005</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>725 BROADWAY</t>
+          <t>23 WYCKOFF AVE</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>WESTWOOD</t>
+          <t>WALDWICK</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -829,12 +829,12 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>ATHLETIC BREWING CO</t>
+          <t>POP SIPS VARIETY 8PK</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>ATHLETIC BREWING COMPANY</t>
+          <t>PASSION TREE</t>
         </is>
       </c>
       <c r="Q4" s="3" t="inlineStr">
@@ -846,17 +846,17 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>09/14/2026 07:35 AM</t>
+          <t>09/15/2026 12:05 PM</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Shane Barreca</t>
+          <t>Mike Ast</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -884,22 +884,22 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>GARDEN STATE DELI (A)</t>
+          <t>WALDWICK WINE/SPIRITS</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>62001</t>
+          <t>88005</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>135 OAKLAND AVE</t>
+          <t>23 WYCKOFF AVE</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>CLOSTER</t>
+          <t>WALDWICK</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -914,12 +914,12 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>CORONA EXTRA</t>
+          <t>COORS LIGHT BEER</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q5" s="3" t="inlineStr">
@@ -931,17 +931,17 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>09/14/2026 07:35 AM</t>
+          <t>09/15/2026 12:05 PM</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>2.2</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Shane Barreca</t>
+          <t>Mike Ast</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -969,22 +969,22 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>GARDEN STATE DELI (A)</t>
+          <t>WALDWICK WINE/SPIRITS</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>62001</t>
+          <t>88005</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>135 OAKLAND AVE</t>
+          <t>23 WYCKOFF AVE</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>CLOSTER</t>
+          <t>WALDWICK</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -999,12 +999,12 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>CORONA LIGHT</t>
+          <t>MILLER LITE BEER</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q6" s="3" t="inlineStr">
@@ -1016,12 +1016,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>09/14/2026 07:35 AM</t>
+          <t>09/14/2026 09:50 AM</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1050,26 +1050,26 @@
         </is>
       </c>
       <c r="H7" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>GARDEN STATE DELI (A)</t>
+          <t>SHOP RITE LIQ (A)HILLSDAL</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>62001</t>
+          <t>73008</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>135 OAKLAND AVE</t>
+          <t>371 BROADWAY</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>CLOSTER</t>
+          <t>HILLSDALE</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -1084,12 +1084,12 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>CORONA PREMIER</t>
+          <t>TWISTED TEA ORIGINAL</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q7" s="3" t="inlineStr">
@@ -1101,12 +1101,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>09/14/2026 07:35 AM</t>
+          <t>09/14/2026 07:38 AM</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1139,22 +1139,22 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>GARDEN STATE DELI (A)</t>
+          <t>WINEMART DISCOUNT</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>62001</t>
+          <t>74005</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>135 OAKLAND AVE</t>
+          <t>700 BROADWAY SUITE 42</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>CLOSTER</t>
+          <t>WESTWOOD</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -1169,12 +1169,12 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>MODELO ESPECIAL</t>
+          <t>NIGHT SHIFT X CAPE MAY BREWBERRY</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>NIGHT SHIFT BREWING</t>
         </is>
       </c>
       <c r="Q8" s="3" t="inlineStr">
@@ -1186,12 +1186,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>09/14/2026 07:31 AM</t>
+          <t>09/14/2026 07:36 AM</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1254,12 +1254,12 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>ATHLETIC BREWING CO</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>ATHLETIC BREWING COMPANY</t>
         </is>
       </c>
       <c r="Q9" s="3" t="inlineStr">
@@ -1271,22 +1271,22 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>09/11/2026 08:55 AM</t>
+          <t>09/14/2026 07:35 AM</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Matthew Powierski</t>
+          <t>Shane Barreca</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Denise Montes</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1309,22 +1309,22 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>HOME WINE LIQUOR (PASSAIC)</t>
+          <t>GARDEN STATE DELI (A)</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>27031</t>
+          <t>62001</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>593 MAIN AVE</t>
+          <t>135 OAKLAND AVE</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>PASSAIC</t>
+          <t>CLOSTER</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
@@ -1339,12 +1339,12 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>KEYSTONE ICE</t>
+          <t>CORONA EXTRA</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q10" s="3" t="inlineStr">
@@ -1356,22 +1356,22 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>09/10/2026 11:46 AM</t>
+          <t>09/14/2026 07:35 AM</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Matthew Powierski</t>
+          <t>Shane Barreca</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Denise Montes</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1394,27 +1394,27 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>WINE GRAND (CARLSTADT)</t>
+          <t>GARDEN STATE DELI (A)</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>32017</t>
+          <t>62001</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>675 PATERSON AVE</t>
+          <t>135 OAKLAND AVE</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>CARLSTADT</t>
+          <t>CLOSTER</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>MBO</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1424,12 +1424,12 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>KEYSTONE ICE</t>
+          <t>CORONA LIGHT</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q11" s="3" t="inlineStr">
@@ -1441,17 +1441,17 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>09/09/2026 12:40 PM</t>
+          <t>09/14/2026 07:35 AM</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>3.3</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Jayson Romine</t>
+          <t>Shane Barreca</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1475,31 +1475,31 @@
         </is>
       </c>
       <c r="H12" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB OF NEWTON (A)</t>
+          <t>GARDEN STATE DELI (A)</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>230412</t>
+          <t>62001</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>17 HAMPTON HOUSE ROAD</t>
+          <t>135 OAKLAND AVE</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>NEWTON</t>
+          <t>CLOSTER</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>MBO</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1509,12 +1509,12 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>ATHLETIC BREWING CO</t>
+          <t>CORONA PREMIER</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>ATHLETIC BREWING COMPANY</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q12" s="3" t="inlineStr">
@@ -1526,17 +1526,17 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>09/09/2026 12:40 PM</t>
+          <t>09/14/2026 07:35 AM</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Jayson Romine</t>
+          <t>Shane Barreca</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1564,27 +1564,27 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB OF NEWTON (A)</t>
+          <t>GARDEN STATE DELI (A)</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>230412</t>
+          <t>62001</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>17 HAMPTON HOUSE ROAD</t>
+          <t>135 OAKLAND AVE</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>NEWTON</t>
+          <t>CLOSTER</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>MBO</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
@@ -1594,12 +1594,12 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>TALKHOUSE ENCORE VARIETY PACK</t>
+          <t>MODELO ESPECIAL</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>TALKHOUSE ENCORE</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q13" s="3" t="inlineStr">
@@ -1611,17 +1611,17 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>09/09/2026 12:40 PM</t>
+          <t>09/14/2026 07:31 AM</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Jayson Romine</t>
+          <t>Shane Barreca</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1649,27 +1649,27 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB OF NEWTON (A)</t>
+          <t>WESTWOOD WINE AND LIQUORS</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>230412</t>
+          <t>74009</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>17 HAMPTON HOUSE ROAD</t>
+          <t>725 BROADWAY</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>NEWTON</t>
+          <t>WESTWOOD</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>MBO</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -1679,12 +1679,12 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISER ICED TEA + VODKA, CLASSIC ICED TEA</t>
+          <t>CAPE MAY BREWING COMPANY</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>CAPE MAY BREWING COMPANY</t>
         </is>
       </c>
       <c r="Q14" s="3" t="inlineStr">
@@ -1696,22 +1696,22 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>09/09/2026 12:40 PM</t>
+          <t>09/11/2026 08:55 AM</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Jayson Romine</t>
+          <t>Matthew Powierski</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1734,27 +1734,27 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB OF NEWTON (A)</t>
+          <t>HOME WINE LIQUOR (PASSAIC)</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>230412</t>
+          <t>27031</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>17 HAMPTON HOUSE ROAD</t>
+          <t>593 MAIN AVE</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>NEWTON</t>
+          <t>PASSAIC</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>MBO</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
@@ -1764,12 +1764,12 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISER ICED TEA + VODKA, HALF &amp; HALF</t>
+          <t>KEYSTONE ICE</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q15" s="3" t="inlineStr">
@@ -1781,22 +1781,22 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>09/09/2026 12:40 PM</t>
+          <t>09/10/2026 11:46 AM</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>8.3</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Jayson Romine</t>
+          <t>Matthew Powierski</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1819,22 +1819,22 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB OF NEWTON (A)</t>
+          <t>WINE GRAND (CARLSTADT)</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>230412</t>
+          <t>32017</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>17 HAMPTON HOUSE ROAD</t>
+          <t>675 PATERSON AVE</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>NEWTON</t>
+          <t>CARLSTADT</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
@@ -1849,12 +1849,12 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISER ICED TEA VODKA VARIETY 18 PACK</t>
+          <t>KEYSTONE ICE</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q16" s="3" t="inlineStr">
@@ -1871,7 +1871,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>8.4</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1900,7 +1900,7 @@
         </is>
       </c>
       <c r="H17" s="2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
@@ -1934,12 +1934,12 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISERS RTD</t>
+          <t>ATHLETIC BREWING CO</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>ATHLETIC BREWING COMPANY</t>
         </is>
       </c>
       <c r="Q17" s="3" t="inlineStr">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1985,7 +1985,7 @@
         </is>
       </c>
       <c r="H18" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
@@ -2019,12 +2019,12 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>TALKHOUSE ENCORE VARIETY PACK</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>TALKHOUSE ENCORE</t>
         </is>
       </c>
       <c r="Q18" s="3" t="inlineStr">
@@ -2036,22 +2036,22 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>09/09/2026 10:37 AM</t>
+          <t>09/09/2026 12:40 PM</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Jayson Romine</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -2074,27 +2074,27 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>WINELAND</t>
+          <t>USA WINE TRADERS CLUB OF NEWTON (A)</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>50020</t>
+          <t>230412</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>247 DEGRAW AVE</t>
+          <t>17 HAMPTON HOUSE ROAD</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>TEANECK</t>
+          <t>NEWTON</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>MBO</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
@@ -2104,10 +2104,14 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>MONACO</t>
-        </is>
-      </c>
-      <c r="P19" s="2" t="n"/>
+          <t>SUN CRUISER ICED TEA + VODKA, CLASSIC ICED TEA</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>BOSTON BEER COMPANY</t>
+        </is>
+      </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
@@ -2117,17 +2121,17 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 12:28 PM</t>
+          <t>09/09/2026 12:40 PM</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Mike Ast</t>
+          <t>Jayson Romine</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -2155,27 +2159,27 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>WALDWICK WINE/SPIRITS</t>
+          <t>USA WINE TRADERS CLUB OF NEWTON (A)</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>88005</t>
+          <t>230412</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>23 WYCKOFF AVE</t>
+          <t>17 HAMPTON HOUSE ROAD</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>WALDWICK</t>
+          <t>NEWTON</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>MBO</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
@@ -2185,7 +2189,7 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISERS RTD</t>
+          <t>SUN CRUISER ICED TEA + VODKA, HALF &amp; HALF</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -2202,17 +2206,17 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 12:28 PM</t>
+          <t>09/09/2026 12:40 PM</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>8.3</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Mike Ast</t>
+          <t>Jayson Romine</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -2240,27 +2244,27 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>WALDWICK WINE/SPIRITS</t>
+          <t>USA WINE TRADERS CLUB OF NEWTON (A)</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>88005</t>
+          <t>230412</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>23 WYCKOFF AVE</t>
+          <t>17 HAMPTON HOUSE ROAD</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>WALDWICK</t>
+          <t>NEWTON</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>MBO</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr">
@@ -2270,12 +2274,12 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>BLUE MOON BELGIAN WHITE ALE</t>
+          <t>SUN CRUISER ICED TEA VODKA VARIETY 18 PACK</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q21" s="3" t="inlineStr">
@@ -2287,22 +2291,22 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 12:17 PM</t>
+          <t>09/09/2026 12:40 PM</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>8.4</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Derrick laws</t>
+          <t>Jayson Romine</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Denise Montes</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -2325,27 +2329,27 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>RAPHAEL &amp; ANGEL LIQ (A)</t>
+          <t>USA WINE TRADERS CLUB OF NEWTON (A)</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>20080</t>
+          <t>230412</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>390 MAIN ST</t>
+          <t>17 HAMPTON HOUSE ROAD</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>PATERSON</t>
+          <t>NEWTON</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>MBO</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr">
@@ -2355,12 +2359,12 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>COORS LIGHT BEER</t>
+          <t>SUN CRUISERS RTD</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q22" s="3" t="inlineStr">
@@ -2372,22 +2376,22 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 11:37 AM</t>
+          <t>09/09/2026 12:40 PM</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Derrick laws</t>
+          <t>Jayson Romine</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Denise Montes</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -2406,31 +2410,31 @@
         </is>
       </c>
       <c r="H23" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>THE LIQUOR SHOP</t>
+          <t>USA WINE TRADERS CLUB OF NEWTON (A)</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>21033</t>
+          <t>230412</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>498 E 30TH STREET</t>
+          <t>17 HAMPTON HOUSE ROAD</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>PATERSON</t>
+          <t>NEWTON</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>MBO</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
@@ -2440,12 +2444,12 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>MODELO CHELADA</t>
+          <t>CAPE MAY BREWING COMPANY</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>CAPE MAY BREWING COMPANY</t>
         </is>
       </c>
       <c r="Q23" s="3" t="inlineStr">
@@ -2457,22 +2461,22 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 11:35 AM</t>
+          <t>09/09/2026 10:37 AM</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Derrick laws</t>
+          <t>Chris Payton</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Denise Montes</t>
+          <t>Michael Engel</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -2495,22 +2499,22 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>THE LIQUOR SHOP</t>
+          <t>WINELAND</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>21033</t>
+          <t>50020</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>498 E 30TH STREET</t>
+          <t>247 DEGRAW AVE</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>PATERSON</t>
+          <t>TEANECK</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
@@ -2525,14 +2529,10 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>CERVEZA REPUBLICA LA TUYA 5.0 LA DURA</t>
-        </is>
-      </c>
-      <c r="P24" s="2" t="inlineStr">
-        <is>
-          <t>VINAIO IMPORTS LTD</t>
-        </is>
-      </c>
+          <t>MONACO</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="n"/>
       <c r="Q24" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
@@ -2542,22 +2542,22 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 11:34 AM</t>
+          <t>09/08/2026 12:28 PM</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Derrick laws</t>
+          <t>Mike Ast</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Denise Montes</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -2580,22 +2580,22 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>THE LIQUOR SHOP</t>
+          <t>WALDWICK WINE/SPIRITS</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>21033</t>
+          <t>88005</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>498 E 30TH STREET</t>
+          <t>23 WYCKOFF AVE</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>PATERSON</t>
+          <t>WALDWICK</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
@@ -2610,12 +2610,12 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>MODELO ORO</t>
+          <t>SUN CRUISERS RTD</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q25" s="3" t="inlineStr">
@@ -2627,22 +2627,22 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 11:32 AM</t>
+          <t>09/08/2026 12:28 PM</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Derrick laws</t>
+          <t>Mike Ast</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Denise Montes</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -2665,22 +2665,22 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>THE LIQUOR SHOP</t>
+          <t>WALDWICK WINE/SPIRITS</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>21033</t>
+          <t>88005</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>498 E 30TH STREET</t>
+          <t>23 WYCKOFF AVE</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>PATERSON</t>
+          <t>WALDWICK</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
@@ -2695,12 +2695,12 @@
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>MODELO ESPECIAL</t>
+          <t>BLUE MOON BELGIAN WHITE ALE</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q26" s="3" t="inlineStr">
@@ -2712,22 +2712,22 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:34 AM</t>
+          <t>09/08/2026 12:17 PM</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Derrick laws</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -2750,22 +2750,22 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
+          <t>RAPHAEL &amp; ANGEL LIQ (A)</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>76010</t>
+          <t>20080</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>66 MARKET ST</t>
+          <t>390 MAIN ST</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>SADDLE BROOK</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
@@ -2780,12 +2780,12 @@
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>CARBLISS</t>
+          <t>COORS LIGHT BEER</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>DRINK CARBLISS</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q27" s="3" t="inlineStr">
@@ -2797,22 +2797,22 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:33 AM</t>
+          <t>09/08/2026 11:37 AM</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Derrick laws</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -2835,22 +2835,22 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
+          <t>THE LIQUOR SHOP</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>76010</t>
+          <t>21033</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>66 MARKET ST</t>
+          <t>498 E 30TH STREET</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>SADDLE BROOK</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
@@ -2865,12 +2865,12 @@
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>TRULY HARD SELTZER</t>
+          <t>MODELO CHELADA</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q28" s="3" t="inlineStr">
@@ -2882,22 +2882,22 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:32 AM</t>
+          <t>09/08/2026 11:35 AM</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Derrick laws</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -2920,22 +2920,22 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
+          <t>THE LIQUOR SHOP</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>76010</t>
+          <t>21033</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>66 MARKET ST</t>
+          <t>498 E 30TH STREET</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>SADDLE BROOK</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
@@ -2950,12 +2950,12 @@
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>COORS LIGHT BEER</t>
+          <t>CERVEZA REPUBLICA LA TUYA 5.0 LA DURA</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>VINAIO IMPORTS LTD</t>
         </is>
       </c>
       <c r="Q29" s="3" t="inlineStr">
@@ -2967,22 +2967,22 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:31 AM</t>
+          <t>09/08/2026 11:34 AM</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Derrick laws</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -3005,22 +3005,22 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
+          <t>THE LIQUOR SHOP</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>76010</t>
+          <t>21033</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>66 MARKET ST</t>
+          <t>498 E 30TH STREET</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>SADDLE BROOK</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
@@ -3035,7 +3035,7 @@
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>CORONA EXTRA</t>
+          <t>MODELO ORO</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
@@ -3052,22 +3052,22 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:31 AM</t>
+          <t>09/08/2026 11:32 AM</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Derrick laws</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -3090,22 +3090,22 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
+          <t>THE LIQUOR SHOP</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>76010</t>
+          <t>21033</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>66 MARKET ST</t>
+          <t>498 E 30TH STREET</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>SADDLE BROOK</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
@@ -3137,12 +3137,12 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:30 AM</t>
+          <t>09/03/2026 11:34 AM</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -3205,12 +3205,12 @@
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>CARBLISS</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>DRINK CARBLISS</t>
         </is>
       </c>
       <c r="Q32" s="3" t="inlineStr">
@@ -3222,12 +3222,12 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:29 AM</t>
+          <t>09/03/2026 11:33 AM</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISERS RTD</t>
+          <t>TRULY HARD SELTZER</t>
         </is>
       </c>
       <c r="P33" s="2" t="inlineStr">
@@ -3307,22 +3307,22 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:11 AM</t>
+          <t>09/03/2026 11:32 AM</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Mike Ast</t>
+          <t>Chris Payton</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
+          <t>Michael Engel</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -3345,22 +3345,22 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>FAIR LAWN WINE &amp; SPIRITS</t>
+          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>81006</t>
+          <t>76010</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>21-00 MAPLE AVE</t>
+          <t>66 MARKET ST</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>FAIR LAWN</t>
+          <t>SADDLE BROOK</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr">
@@ -3375,12 +3375,12 @@
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISERS RTD</t>
+          <t>COORS LIGHT BEER</t>
         </is>
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q34" s="3" t="inlineStr">
@@ -3392,12 +3392,12 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 10:31 AM</t>
+          <t>09/03/2026 11:31 AM</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -3430,22 +3430,22 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON DISC LIQ (A)</t>
+          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>25045</t>
+          <t>76010</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>73 ACKERMAN AVE BOTONY PL</t>
+          <t>66 MARKET ST</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON</t>
+          <t>SADDLE BROOK</t>
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr">
@@ -3460,12 +3460,12 @@
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>CARBLISS</t>
+          <t>CORONA EXTRA</t>
         </is>
       </c>
       <c r="P35" s="2" t="inlineStr">
         <is>
-          <t>DRINK CARBLISS</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q35" s="3" t="inlineStr">
@@ -3477,12 +3477,12 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 10:30 AM</t>
+          <t>09/03/2026 11:31 AM</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -3515,22 +3515,22 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON DISC LIQ (A)</t>
+          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>25045</t>
+          <t>76010</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>73 ACKERMAN AVE BOTONY PL</t>
+          <t>66 MARKET ST</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON</t>
+          <t>SADDLE BROOK</t>
         </is>
       </c>
       <c r="M36" s="2" t="inlineStr">
@@ -3545,7 +3545,7 @@
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>CORONA EXTRA</t>
+          <t>MODELO ESPECIAL</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
@@ -3562,12 +3562,12 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 10:29 AM</t>
+          <t>09/03/2026 11:30 AM</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -3600,22 +3600,22 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON DISC LIQ (A)</t>
+          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>25045</t>
+          <t>76010</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>73 ACKERMAN AVE BOTONY PL</t>
+          <t>66 MARKET ST</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON</t>
+          <t>SADDLE BROOK</t>
         </is>
       </c>
       <c r="M37" s="2" t="inlineStr">
@@ -3630,12 +3630,12 @@
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>MODELO ESPECIAL</t>
+          <t>CAPE MAY BREWING COMPANY</t>
         </is>
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>CAPE MAY BREWING COMPANY</t>
         </is>
       </c>
       <c r="Q37" s="3" t="inlineStr">
@@ -3647,12 +3647,12 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 10:28 AM</t>
+          <t>09/03/2026 11:29 AM</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -3685,22 +3685,22 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON DISC LIQ (A)</t>
+          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>25045</t>
+          <t>76010</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>73 ACKERMAN AVE BOTONY PL</t>
+          <t>66 MARKET ST</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON</t>
+          <t>SADDLE BROOK</t>
         </is>
       </c>
       <c r="M38" s="2" t="inlineStr">
@@ -3715,12 +3715,12 @@
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>COORS LIGHT BEER</t>
+          <t>SUN CRUISERS RTD</t>
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q38" s="3" t="inlineStr">
@@ -3732,22 +3732,22 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 10:28 AM</t>
+          <t>09/03/2026 11:11 AM</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Mike Ast</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -3770,22 +3770,22 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON DISC LIQ (A)</t>
+          <t>FAIR LAWN WINE &amp; SPIRITS</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>25045</t>
+          <t>81006</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>73 ACKERMAN AVE BOTONY PL</t>
+          <t>21-00 MAPLE AVE</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON</t>
+          <t>FAIR LAWN</t>
         </is>
       </c>
       <c r="M39" s="2" t="inlineStr">
@@ -3800,12 +3800,12 @@
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>MILLER LITE BEER</t>
+          <t>SUN CRUISERS RTD</t>
         </is>
       </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q39" s="3" t="inlineStr">
@@ -3817,83 +3817,508 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
+          <t>09/03/2026 10:31 AM</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>8.1</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Chris Payton</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Michael Engel</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON DISC LIQ (A)</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>25045</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>73 ACKERMAN AVE BOTONY PL</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>MBO</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>Cooler Door Wrap</t>
+        </is>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>CARBLISS</t>
+        </is>
+      </c>
+      <c r="P40" s="2" t="inlineStr">
+        <is>
+          <t>DRINK CARBLISS</t>
+        </is>
+      </c>
+      <c r="Q40" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>09/03/2026 10:30 AM</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Chris Payton</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Michael Engel</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON DISC LIQ (A)</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>25045</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>73 ACKERMAN AVE BOTONY PL</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>MBO</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="inlineStr">
+        <is>
+          <t>Cooler Door Wrap</t>
+        </is>
+      </c>
+      <c r="O41" s="2" t="inlineStr">
+        <is>
+          <t>CORONA EXTRA</t>
+        </is>
+      </c>
+      <c r="P41" s="2" t="inlineStr">
+        <is>
+          <t>CONSTELLATION BRANDS</t>
+        </is>
+      </c>
+      <c r="Q41" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>09/03/2026 10:29 AM</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>10.1</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Chris Payton</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Michael Engel</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON DISC LIQ (A)</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>25045</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>73 ACKERMAN AVE BOTONY PL</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>MBO</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>Cooler Door Wrap</t>
+        </is>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>MODELO ESPECIAL</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="inlineStr">
+        <is>
+          <t>CONSTELLATION BRANDS</t>
+        </is>
+      </c>
+      <c r="Q42" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>09/03/2026 10:28 AM</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>11.1</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Chris Payton</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Michael Engel</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON DISC LIQ (A)</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>25045</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>73 ACKERMAN AVE BOTONY PL</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON</t>
+        </is>
+      </c>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>MBO</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
+          <t>Cooler Door Wrap</t>
+        </is>
+      </c>
+      <c r="O43" s="2" t="inlineStr">
+        <is>
+          <t>COORS LIGHT BEER</t>
+        </is>
+      </c>
+      <c r="P43" s="2" t="inlineStr">
+        <is>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
+        </is>
+      </c>
+      <c r="Q43" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>09/03/2026 10:28 AM</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>11.2</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Chris Payton</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Michael Engel</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON DISC LIQ (A)</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>25045</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>73 ACKERMAN AVE BOTONY PL</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>MBO</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>Cooler Door Wrap</t>
+        </is>
+      </c>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>MILLER LITE BEER</t>
+        </is>
+      </c>
+      <c r="P44" s="2" t="inlineStr">
+        <is>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
+        </is>
+      </c>
+      <c r="Q44" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
           <t>09/03/2026 10:27 AM</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B45" s="2" t="inlineStr">
         <is>
           <t>12.1</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr">
         <is>
           <t>Chris Payton</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>Michael Engel</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E45" s="2" t="inlineStr">
         <is>
           <t>Ashley Furman</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="F45" s="2" t="inlineStr">
         <is>
           <t>Sales Rep</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G45" s="2" t="inlineStr">
         <is>
           <t>Feature Activation</t>
         </is>
       </c>
-      <c r="H40" s="2" t="n">
+      <c r="H45" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="I40" s="2" t="inlineStr">
+      <c r="I45" s="2" t="inlineStr">
         <is>
           <t>CLIFTON DISC LIQ (A)</t>
         </is>
       </c>
-      <c r="J40" s="2" t="inlineStr">
+      <c r="J45" s="2" t="inlineStr">
         <is>
           <t>25045</t>
         </is>
       </c>
-      <c r="K40" s="2" t="inlineStr">
+      <c r="K45" s="2" t="inlineStr">
         <is>
           <t>73 ACKERMAN AVE BOTONY PL</t>
         </is>
       </c>
-      <c r="L40" s="2" t="inlineStr">
+      <c r="L45" s="2" t="inlineStr">
         <is>
           <t>CLIFTON</t>
         </is>
       </c>
-      <c r="M40" s="2" t="inlineStr">
+      <c r="M45" s="2" t="inlineStr">
         <is>
           <t>MBO</t>
         </is>
       </c>
-      <c r="N40" s="2" t="inlineStr">
+      <c r="N45" s="2" t="inlineStr">
         <is>
           <t>Cooler Door Wrap</t>
         </is>
       </c>
-      <c r="O40" s="2" t="inlineStr">
+      <c r="O45" s="2" t="inlineStr">
         <is>
           <t>MODELO CHELADA</t>
         </is>
       </c>
-      <c r="P40" s="2" t="inlineStr">
+      <c r="P45" s="2" t="inlineStr">
         <is>
           <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
-      <c r="Q40" s="3" t="inlineStr">
+      <c r="Q45" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
         </is>
@@ -3940,6 +4365,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q38" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId44"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Off-prem MPO: Promos_Report_25 merged into the cooler-door archive (33 -> 34 stickers)
45 rows, all Cooler Door Wrap, 1 new: Matt Powierski's Keystone Ice wrap at
Metro Liquors (East Rutherford), 9/16, taking him 2 -> 3. Archive 44 -> 45
rows, photo links intact; still 4 reps at goal. Nothing else re-pulled.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EWaRBkSPoZwPoGXmdfLY6t
</commit_message>
<xml_diff>
--- a/MPOs/off-prem/pos_cooler_door_promos.xlsx
+++ b/MPOs/off-prem/pos_cooler_door_promos.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q45"/>
+  <dimension ref="A1:Q46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21.7109375" customWidth="1" style="6" min="1" max="1"/>
@@ -591,7 +591,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>09/15/2026 12:07 PM</t>
+          <t>09/16/2026 01:16 PM</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -601,12 +601,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Mike Ast</t>
+          <t>Matthew Powierski</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -629,22 +629,22 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>WALDWICK WINE/SPIRITS</t>
+          <t>METRO LIQUORS (EAST RUTHERFORD)</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>88005</t>
+          <t>31004</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>23 WYCKOFF AVE</t>
+          <t>576 PATERSON AVE</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>WALDWICK</t>
+          <t>EAST RUTHERFORD</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -659,12 +659,12 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>POP SIPS GINGER LIME</t>
+          <t>KEYSTONE ICE</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>PASSION TREE</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q2" s="3" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -744,7 +744,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>POP SIPS RASPBERRY ROSE</t>
+          <t>POP SIPS GINGER LIME</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -766,7 +766,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -829,7 +829,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>POP SIPS VARIETY 8PK</t>
+          <t>POP SIPS RASPBERRY ROSE</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -846,12 +846,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>09/15/2026 12:05 PM</t>
+          <t>09/15/2026 12:07 PM</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -914,12 +914,12 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>COORS LIGHT BEER</t>
+          <t>POP SIPS VARIETY 8PK</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>PASSION TREE</t>
         </is>
       </c>
       <c r="Q5" s="3" t="inlineStr">
@@ -936,7 +936,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -999,7 +999,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>MILLER LITE BEER</t>
+          <t>COORS LIGHT BEER</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1016,17 +1016,17 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>09/14/2026 09:50 AM</t>
+          <t>09/15/2026 12:05 PM</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>2.2</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Shane Barreca</t>
+          <t>Mike Ast</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -1050,26 +1050,26 @@
         </is>
       </c>
       <c r="H7" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>SHOP RITE LIQ (A)HILLSDAL</t>
+          <t>WALDWICK WINE/SPIRITS</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>73008</t>
+          <t>88005</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>371 BROADWAY</t>
+          <t>23 WYCKOFF AVE</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>HILLSDALE</t>
+          <t>WALDWICK</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -1084,12 +1084,12 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>TWISTED TEA ORIGINAL</t>
+          <t>MILLER LITE BEER</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q7" s="3" t="inlineStr">
@@ -1101,7 +1101,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>09/14/2026 07:38 AM</t>
+          <t>09/14/2026 09:50 AM</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1135,26 +1135,26 @@
         </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>WINEMART DISCOUNT</t>
+          <t>SHOP RITE LIQ (A)HILLSDAL</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>74005</t>
+          <t>73008</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>700 BROADWAY SUITE 42</t>
+          <t>371 BROADWAY</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>WESTWOOD</t>
+          <t>HILLSDALE</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -1169,12 +1169,12 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>NIGHT SHIFT X CAPE MAY BREWBERRY</t>
+          <t>TWISTED TEA ORIGINAL</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>NIGHT SHIFT BREWING</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q8" s="3" t="inlineStr">
@@ -1186,12 +1186,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>09/14/2026 07:36 AM</t>
+          <t>09/14/2026 07:38 AM</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1224,17 +1224,17 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>WESTWOOD WINE AND LIQUORS</t>
+          <t>WINEMART DISCOUNT</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>74009</t>
+          <t>74005</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>725 BROADWAY</t>
+          <t>700 BROADWAY SUITE 42</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1254,12 +1254,12 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>ATHLETIC BREWING CO</t>
+          <t>NIGHT SHIFT X CAPE MAY BREWBERRY</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>ATHLETIC BREWING COMPANY</t>
+          <t>NIGHT SHIFT BREWING</t>
         </is>
       </c>
       <c r="Q9" s="3" t="inlineStr">
@@ -1271,12 +1271,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>09/14/2026 07:35 AM</t>
+          <t>09/14/2026 07:36 AM</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1309,22 +1309,22 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>GARDEN STATE DELI (A)</t>
+          <t>WESTWOOD WINE AND LIQUORS</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>62001</t>
+          <t>74009</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>135 OAKLAND AVE</t>
+          <t>725 BROADWAY</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>CLOSTER</t>
+          <t>WESTWOOD</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
@@ -1339,12 +1339,12 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>CORONA EXTRA</t>
+          <t>ATHLETIC BREWING CO</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>ATHLETIC BREWING COMPANY</t>
         </is>
       </c>
       <c r="Q10" s="3" t="inlineStr">
@@ -1361,7 +1361,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>CORONA LIGHT</t>
+          <t>CORONA EXTRA</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1509,7 +1509,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>CORONA PREMIER</t>
+          <t>CORONA LIGHT</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>3.3</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>MODELO ESPECIAL</t>
+          <t>CORONA PREMIER</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -1611,12 +1611,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>09/14/2026 07:31 AM</t>
+          <t>09/14/2026 07:35 AM</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1649,22 +1649,22 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>WESTWOOD WINE AND LIQUORS</t>
+          <t>GARDEN STATE DELI (A)</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>74009</t>
+          <t>62001</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>725 BROADWAY</t>
+          <t>135 OAKLAND AVE</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>WESTWOOD</t>
+          <t>CLOSTER</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
@@ -1679,12 +1679,12 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>MODELO ESPECIAL</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q14" s="3" t="inlineStr">
@@ -1696,22 +1696,22 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>09/11/2026 08:55 AM</t>
+          <t>09/14/2026 07:31 AM</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Matthew Powierski</t>
+          <t>Shane Barreca</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Denise Montes</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1734,22 +1734,22 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>HOME WINE LIQUOR (PASSAIC)</t>
+          <t>WESTWOOD WINE AND LIQUORS</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>27031</t>
+          <t>74009</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>593 MAIN AVE</t>
+          <t>725 BROADWAY</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>PASSAIC</t>
+          <t>WESTWOOD</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
@@ -1764,12 +1764,12 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>KEYSTONE ICE</t>
+          <t>CAPE MAY BREWING COMPANY</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>CAPE MAY BREWING COMPANY</t>
         </is>
       </c>
       <c r="Q15" s="3" t="inlineStr">
@@ -1781,12 +1781,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>09/10/2026 11:46 AM</t>
+          <t>09/11/2026 08:55 AM</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1819,27 +1819,27 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>WINE GRAND (CARLSTADT)</t>
+          <t>HOME WINE LIQUOR (PASSAIC)</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>32017</t>
+          <t>27031</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>675 PATERSON AVE</t>
+          <t>593 MAIN AVE</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>CARLSTADT</t>
+          <t>PASSAIC</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>MBO</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -1866,22 +1866,22 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>09/09/2026 12:40 PM</t>
+          <t>09/10/2026 11:46 AM</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Jayson Romine</t>
+          <t>Matthew Powierski</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1900,26 +1900,26 @@
         </is>
       </c>
       <c r="H17" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB OF NEWTON (A)</t>
+          <t>WINE GRAND (CARLSTADT)</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>230412</t>
+          <t>32017</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>17 HAMPTON HOUSE ROAD</t>
+          <t>675 PATERSON AVE</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>NEWTON</t>
+          <t>CARLSTADT</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
@@ -1934,12 +1934,12 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>ATHLETIC BREWING CO</t>
+          <t>KEYSTONE ICE</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>ATHLETIC BREWING COMPANY</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q17" s="3" t="inlineStr">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1985,7 +1985,7 @@
         </is>
       </c>
       <c r="H18" s="2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
@@ -2019,12 +2019,12 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>TALKHOUSE ENCORE VARIETY PACK</t>
+          <t>ATHLETIC BREWING CO</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>TALKHOUSE ENCORE</t>
+          <t>ATHLETIC BREWING COMPANY</t>
         </is>
       </c>
       <c r="Q18" s="3" t="inlineStr">
@@ -2041,7 +2041,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -2104,12 +2104,12 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISER ICED TEA + VODKA, CLASSIC ICED TEA</t>
+          <t>TALKHOUSE ENCORE VARIETY PACK</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>TALKHOUSE ENCORE</t>
         </is>
       </c>
       <c r="Q19" s="3" t="inlineStr">
@@ -2126,7 +2126,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISER ICED TEA + VODKA, HALF &amp; HALF</t>
+          <t>SUN CRUISER ICED TEA + VODKA, CLASSIC ICED TEA</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -2211,7 +2211,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>8.3</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -2274,7 +2274,7 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISER ICED TEA VODKA VARIETY 18 PACK</t>
+          <t>SUN CRUISER ICED TEA + VODKA, HALF &amp; HALF</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
@@ -2296,7 +2296,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>8.4</t>
+          <t>8.3</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -2359,7 +2359,7 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISERS RTD</t>
+          <t>SUN CRUISER ICED TEA VODKA VARIETY 18 PACK</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>8.4</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -2410,7 +2410,7 @@
         </is>
       </c>
       <c r="H23" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
@@ -2444,12 +2444,12 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>SUN CRUISERS RTD</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q23" s="3" t="inlineStr">
@@ -2461,22 +2461,22 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>09/09/2026 10:37 AM</t>
+          <t>09/09/2026 12:40 PM</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Jayson Romine</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -2495,31 +2495,31 @@
         </is>
       </c>
       <c r="H24" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>WINELAND</t>
+          <t>USA WINE TRADERS CLUB OF NEWTON (A)</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>50020</t>
+          <t>230412</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>247 DEGRAW AVE</t>
+          <t>17 HAMPTON HOUSE ROAD</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>TEANECK</t>
+          <t>NEWTON</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>MBO</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
@@ -2529,10 +2529,14 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>MONACO</t>
-        </is>
-      </c>
-      <c r="P24" s="2" t="n"/>
+          <t>CAPE MAY BREWING COMPANY</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>CAPE MAY BREWING COMPANY</t>
+        </is>
+      </c>
       <c r="Q24" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
@@ -2542,22 +2546,22 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 12:28 PM</t>
+          <t>09/09/2026 10:37 AM</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Mike Ast</t>
+          <t>Chris Payton</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
+          <t>Michael Engel</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -2580,22 +2584,22 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>WALDWICK WINE/SPIRITS</t>
+          <t>WINELAND</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>88005</t>
+          <t>50020</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>23 WYCKOFF AVE</t>
+          <t>247 DEGRAW AVE</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>WALDWICK</t>
+          <t>TEANECK</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
@@ -2610,14 +2614,10 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISERS RTD</t>
-        </is>
-      </c>
-      <c r="P25" s="2" t="inlineStr">
-        <is>
-          <t>BOSTON BEER COMPANY</t>
-        </is>
-      </c>
+          <t>MONACO</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="n"/>
       <c r="Q25" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
@@ -2632,7 +2632,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -2695,12 +2695,12 @@
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>BLUE MOON BELGIAN WHITE ALE</t>
+          <t>SUN CRUISERS RTD</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q26" s="3" t="inlineStr">
@@ -2712,22 +2712,22 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 12:17 PM</t>
+          <t>09/08/2026 12:28 PM</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Derrick laws</t>
+          <t>Mike Ast</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Denise Montes</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -2750,22 +2750,22 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>RAPHAEL &amp; ANGEL LIQ (A)</t>
+          <t>WALDWICK WINE/SPIRITS</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>20080</t>
+          <t>88005</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>390 MAIN ST</t>
+          <t>23 WYCKOFF AVE</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>PATERSON</t>
+          <t>WALDWICK</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
@@ -2780,7 +2780,7 @@
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>COORS LIGHT BEER</t>
+          <t>BLUE MOON BELGIAN WHITE ALE</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
@@ -2797,12 +2797,12 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 11:37 AM</t>
+          <t>09/08/2026 12:17 PM</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -2835,17 +2835,17 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>THE LIQUOR SHOP</t>
+          <t>RAPHAEL &amp; ANGEL LIQ (A)</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>21033</t>
+          <t>20080</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>498 E 30TH STREET</t>
+          <t>390 MAIN ST</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
@@ -2865,12 +2865,12 @@
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>MODELO CHELADA</t>
+          <t>COORS LIGHT BEER</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q28" s="3" t="inlineStr">
@@ -2882,12 +2882,12 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 11:35 AM</t>
+          <t>09/08/2026 11:37 AM</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -2950,12 +2950,12 @@
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>CERVEZA REPUBLICA LA TUYA 5.0 LA DURA</t>
+          <t>MODELO CHELADA</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>VINAIO IMPORTS LTD</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q29" s="3" t="inlineStr">
@@ -2967,12 +2967,12 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 11:34 AM</t>
+          <t>09/08/2026 11:35 AM</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -3035,12 +3035,12 @@
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>MODELO ORO</t>
+          <t>CERVEZA REPUBLICA LA TUYA 5.0 LA DURA</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>VINAIO IMPORTS LTD</t>
         </is>
       </c>
       <c r="Q30" s="3" t="inlineStr">
@@ -3052,12 +3052,12 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 11:32 AM</t>
+          <t>09/08/2026 11:34 AM</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>MODELO ESPECIAL</t>
+          <t>MODELO ORO</t>
         </is>
       </c>
       <c r="P31" s="2" t="inlineStr">
@@ -3137,22 +3137,22 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:34 AM</t>
+          <t>09/08/2026 11:32 AM</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Derrick laws</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -3175,22 +3175,22 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
+          <t>THE LIQUOR SHOP</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>76010</t>
+          <t>21033</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>66 MARKET ST</t>
+          <t>498 E 30TH STREET</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>SADDLE BROOK</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
@@ -3205,12 +3205,12 @@
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>CARBLISS</t>
+          <t>MODELO ESPECIAL</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>DRINK CARBLISS</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q32" s="3" t="inlineStr">
@@ -3222,12 +3222,12 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:33 AM</t>
+          <t>09/03/2026 11:34 AM</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -3290,12 +3290,12 @@
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>TRULY HARD SELTZER</t>
+          <t>CARBLISS</t>
         </is>
       </c>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>DRINK CARBLISS</t>
         </is>
       </c>
       <c r="Q33" s="3" t="inlineStr">
@@ -3307,12 +3307,12 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:32 AM</t>
+          <t>09/03/2026 11:33 AM</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -3375,12 +3375,12 @@
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>COORS LIGHT BEER</t>
+          <t>TRULY HARD SELTZER</t>
         </is>
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q34" s="3" t="inlineStr">
@@ -3392,12 +3392,12 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:31 AM</t>
+          <t>09/03/2026 11:32 AM</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -3460,12 +3460,12 @@
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>CORONA EXTRA</t>
+          <t>COORS LIGHT BEER</t>
         </is>
       </c>
       <c r="P35" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q35" s="3" t="inlineStr">
@@ -3482,7 +3482,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -3545,7 +3545,7 @@
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>MODELO ESPECIAL</t>
+          <t>CORONA EXTRA</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
@@ -3562,12 +3562,12 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:30 AM</t>
+          <t>09/03/2026 11:31 AM</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -3630,12 +3630,12 @@
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>MODELO ESPECIAL</t>
         </is>
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q37" s="3" t="inlineStr">
@@ -3647,12 +3647,12 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:29 AM</t>
+          <t>09/03/2026 11:30 AM</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -3715,12 +3715,12 @@
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISERS RTD</t>
+          <t>CAPE MAY BREWING COMPANY</t>
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>CAPE MAY BREWING COMPANY</t>
         </is>
       </c>
       <c r="Q38" s="3" t="inlineStr">
@@ -3732,22 +3732,22 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:11 AM</t>
+          <t>09/03/2026 11:29 AM</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Mike Ast</t>
+          <t>Chris Payton</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
+          <t>Michael Engel</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -3770,22 +3770,22 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>FAIR LAWN WINE &amp; SPIRITS</t>
+          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>81006</t>
+          <t>76010</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>21-00 MAPLE AVE</t>
+          <t>66 MARKET ST</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>FAIR LAWN</t>
+          <t>SADDLE BROOK</t>
         </is>
       </c>
       <c r="M39" s="2" t="inlineStr">
@@ -3817,22 +3817,22 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 10:31 AM</t>
+          <t>09/03/2026 11:11 AM</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Mike Ast</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -3855,22 +3855,22 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON DISC LIQ (A)</t>
+          <t>FAIR LAWN WINE &amp; SPIRITS</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>25045</t>
+          <t>81006</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>73 ACKERMAN AVE BOTONY PL</t>
+          <t>21-00 MAPLE AVE</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON</t>
+          <t>FAIR LAWN</t>
         </is>
       </c>
       <c r="M40" s="2" t="inlineStr">
@@ -3885,12 +3885,12 @@
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>CARBLISS</t>
+          <t>SUN CRUISERS RTD</t>
         </is>
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>DRINK CARBLISS</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q40" s="3" t="inlineStr">
@@ -3902,12 +3902,12 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 10:30 AM</t>
+          <t>09/03/2026 10:31 AM</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -3970,12 +3970,12 @@
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>CORONA EXTRA</t>
+          <t>CARBLISS</t>
         </is>
       </c>
       <c r="P41" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>DRINK CARBLISS</t>
         </is>
       </c>
       <c r="Q41" s="3" t="inlineStr">
@@ -3987,12 +3987,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 10:29 AM</t>
+          <t>09/03/2026 10:30 AM</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -4055,7 +4055,7 @@
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>MODELO ESPECIAL</t>
+          <t>CORONA EXTRA</t>
         </is>
       </c>
       <c r="P42" s="2" t="inlineStr">
@@ -4072,12 +4072,12 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 10:28 AM</t>
+          <t>09/03/2026 10:29 AM</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -4140,12 +4140,12 @@
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>COORS LIGHT BEER</t>
+          <t>MODELO ESPECIAL</t>
         </is>
       </c>
       <c r="P43" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q43" s="3" t="inlineStr">
@@ -4162,7 +4162,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -4225,7 +4225,7 @@
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>MILLER LITE BEER</t>
+          <t>COORS LIGHT BEER</t>
         </is>
       </c>
       <c r="P44" s="2" t="inlineStr">
@@ -4242,83 +4242,168 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
+          <t>09/03/2026 10:28 AM</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>11.2</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Chris Payton</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Michael Engel</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON DISC LIQ (A)</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>25045</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>73 ACKERMAN AVE BOTONY PL</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON</t>
+        </is>
+      </c>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>MBO</t>
+        </is>
+      </c>
+      <c r="N45" s="2" t="inlineStr">
+        <is>
+          <t>Cooler Door Wrap</t>
+        </is>
+      </c>
+      <c r="O45" s="2" t="inlineStr">
+        <is>
+          <t>MILLER LITE BEER</t>
+        </is>
+      </c>
+      <c r="P45" s="2" t="inlineStr">
+        <is>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
+        </is>
+      </c>
+      <c r="Q45" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
           <t>09/03/2026 10:27 AM</t>
         </is>
       </c>
-      <c r="B45" s="2" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>12.1</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>Chris Payton</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>Michael Engel</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>Ashley Furman</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>Sales Rep</t>
         </is>
       </c>
-      <c r="G45" s="2" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>Feature Activation</t>
         </is>
       </c>
-      <c r="H45" s="2" t="n">
+      <c r="H46" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="I45" s="2" t="inlineStr">
+      <c r="I46" s="2" t="inlineStr">
         <is>
           <t>CLIFTON DISC LIQ (A)</t>
         </is>
       </c>
-      <c r="J45" s="2" t="inlineStr">
+      <c r="J46" s="2" t="inlineStr">
         <is>
           <t>25045</t>
         </is>
       </c>
-      <c r="K45" s="2" t="inlineStr">
+      <c r="K46" s="2" t="inlineStr">
         <is>
           <t>73 ACKERMAN AVE BOTONY PL</t>
         </is>
       </c>
-      <c r="L45" s="2" t="inlineStr">
+      <c r="L46" s="2" t="inlineStr">
         <is>
           <t>CLIFTON</t>
         </is>
       </c>
-      <c r="M45" s="2" t="inlineStr">
+      <c r="M46" s="2" t="inlineStr">
         <is>
           <t>MBO</t>
         </is>
       </c>
-      <c r="N45" s="2" t="inlineStr">
+      <c r="N46" s="2" t="inlineStr">
         <is>
           <t>Cooler Door Wrap</t>
         </is>
       </c>
-      <c r="O45" s="2" t="inlineStr">
+      <c r="O46" s="2" t="inlineStr">
         <is>
           <t>MODELO CHELADA</t>
         </is>
       </c>
-      <c r="P45" s="2" t="inlineStr">
+      <c r="P46" s="2" t="inlineStr">
         <is>
           <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
-      <c r="Q45" s="3" t="inlineStr">
+      <c r="Q46" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
         </is>
@@ -4370,6 +4455,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q43" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId45"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Off-prem MPO 9/18 refresh (+ Keystone, Corona Gaintain sync)
Constellation, Keystone, Fever Tree and Wine & Spirits RDE exports
pulled 9/18 onto the September off-prem board, plus Promos_Report_28
merged into the cooler-door archive (1 new sticker row, 45 already
published). Fever Tree 103 -> 124 (Chris Payton and Phil Ernst reach
10), Wine & Spirits 259 -> 290 (Javier Melo and Matt Powierski reach
5), Keystone 166 -> 168 accounts, Constellation 1,043 -> 1,059.

Phil Ernst's 32 rows dated 9/30 at USA Wine Traders Paramus are kept
as every future-dated row has been, and flagged in the README.

Shared exports synced per the sync rule: Keystone onto
keystone-ice/actuals.csv and Corona Gaintain onto the incentive
tracker; both rebuilt. Hub cache tag bumped to 20260918b.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A7q8T2fFHgWKc5RLHMksaS
</commit_message>
<xml_diff>
--- a/MPOs/off-prem/pos_cooler_door_promos.xlsx
+++ b/MPOs/off-prem/pos_cooler_door_promos.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q46"/>
+  <dimension ref="A1:Q47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21.7109375" customWidth="1" style="6" min="1" max="1"/>
@@ -591,7 +591,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 01:16 PM</t>
+          <t>09/17/2026 12:44 PM</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -601,7 +601,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Matthew Powierski</t>
+          <t>Pablo Lopez</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -629,27 +629,27 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>METRO LIQUORS (EAST RUTHERFORD)</t>
+          <t>INTENSITY LOUNGE/ANGIE'S LIQUORS</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>31004</t>
+          <t>20062</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>576 PATERSON AVE</t>
+          <t>109 MAIN ST</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>EAST RUTHERFORD</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>MBO</t>
+          <t>Incentive</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -676,7 +676,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>09/15/2026 12:07 PM</t>
+          <t>09/16/2026 01:16 PM</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -686,12 +686,12 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Mike Ast</t>
+          <t>Matthew Powierski</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -714,22 +714,22 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>WALDWICK WINE/SPIRITS</t>
+          <t>METRO LIQUORS (EAST RUTHERFORD)</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>88005</t>
+          <t>31004</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>23 WYCKOFF AVE</t>
+          <t>576 PATERSON AVE</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>WALDWICK</t>
+          <t>EAST RUTHERFORD</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -744,12 +744,12 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>POP SIPS GINGER LIME</t>
+          <t>KEYSTONE ICE</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>PASSION TREE</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q3" s="3" t="inlineStr">
@@ -766,7 +766,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -829,7 +829,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>POP SIPS RASPBERRY ROSE</t>
+          <t>POP SIPS GINGER LIME</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -851,7 +851,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -914,7 +914,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>POP SIPS VARIETY 8PK</t>
+          <t>POP SIPS RASPBERRY ROSE</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -931,12 +931,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>09/15/2026 12:05 PM</t>
+          <t>09/15/2026 12:07 PM</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -999,12 +999,12 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>COORS LIGHT BEER</t>
+          <t>POP SIPS VARIETY 8PK</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>PASSION TREE</t>
         </is>
       </c>
       <c r="Q6" s="3" t="inlineStr">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1084,7 +1084,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>MILLER LITE BEER</t>
+          <t>COORS LIGHT BEER</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1101,17 +1101,17 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>09/14/2026 09:50 AM</t>
+          <t>09/15/2026 12:05 PM</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>2.2</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Shane Barreca</t>
+          <t>Mike Ast</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1135,26 +1135,26 @@
         </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>SHOP RITE LIQ (A)HILLSDAL</t>
+          <t>WALDWICK WINE/SPIRITS</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>73008</t>
+          <t>88005</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>371 BROADWAY</t>
+          <t>23 WYCKOFF AVE</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>HILLSDALE</t>
+          <t>WALDWICK</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -1169,12 +1169,12 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>TWISTED TEA ORIGINAL</t>
+          <t>MILLER LITE BEER</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q8" s="3" t="inlineStr">
@@ -1186,7 +1186,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>09/14/2026 07:38 AM</t>
+          <t>09/14/2026 09:50 AM</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1220,26 +1220,26 @@
         </is>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>WINEMART DISCOUNT</t>
+          <t>SHOP RITE LIQ (A)HILLSDAL</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>74005</t>
+          <t>73008</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>700 BROADWAY SUITE 42</t>
+          <t>371 BROADWAY</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>WESTWOOD</t>
+          <t>HILLSDALE</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
@@ -1254,12 +1254,12 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>NIGHT SHIFT X CAPE MAY BREWBERRY</t>
+          <t>TWISTED TEA ORIGINAL</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>NIGHT SHIFT BREWING</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q9" s="3" t="inlineStr">
@@ -1271,12 +1271,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>09/14/2026 07:36 AM</t>
+          <t>09/14/2026 07:38 AM</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1309,17 +1309,17 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>WESTWOOD WINE AND LIQUORS</t>
+          <t>WINEMART DISCOUNT</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>74009</t>
+          <t>74005</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>725 BROADWAY</t>
+          <t>700 BROADWAY SUITE 42</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1339,12 +1339,12 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>ATHLETIC BREWING CO</t>
+          <t>NIGHT SHIFT X CAPE MAY BREWBERRY</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>ATHLETIC BREWING COMPANY</t>
+          <t>NIGHT SHIFT BREWING</t>
         </is>
       </c>
       <c r="Q10" s="3" t="inlineStr">
@@ -1356,12 +1356,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>09/14/2026 07:35 AM</t>
+          <t>09/14/2026 07:36 AM</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1394,22 +1394,22 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>GARDEN STATE DELI (A)</t>
+          <t>WESTWOOD WINE AND LIQUORS</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>62001</t>
+          <t>74009</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>135 OAKLAND AVE</t>
+          <t>725 BROADWAY</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>CLOSTER</t>
+          <t>WESTWOOD</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
@@ -1424,12 +1424,12 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>CORONA EXTRA</t>
+          <t>ATHLETIC BREWING CO</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>ATHLETIC BREWING COMPANY</t>
         </is>
       </c>
       <c r="Q11" s="3" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1509,7 +1509,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>CORONA LIGHT</t>
+          <t>CORONA EXTRA</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>CORONA PREMIER</t>
+          <t>CORONA LIGHT</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -1616,7 +1616,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>3.3</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1679,7 +1679,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>MODELO ESPECIAL</t>
+          <t>CORONA PREMIER</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -1696,12 +1696,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>09/14/2026 07:31 AM</t>
+          <t>09/14/2026 07:35 AM</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1734,22 +1734,22 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>WESTWOOD WINE AND LIQUORS</t>
+          <t>GARDEN STATE DELI (A)</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>74009</t>
+          <t>62001</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>725 BROADWAY</t>
+          <t>135 OAKLAND AVE</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>WESTWOOD</t>
+          <t>CLOSTER</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
@@ -1764,12 +1764,12 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>MODELO ESPECIAL</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q15" s="3" t="inlineStr">
@@ -1781,22 +1781,22 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>09/11/2026 08:55 AM</t>
+          <t>09/14/2026 07:31 AM</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Matthew Powierski</t>
+          <t>Shane Barreca</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Denise Montes</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1819,22 +1819,22 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>HOME WINE LIQUOR (PASSAIC)</t>
+          <t>WESTWOOD WINE AND LIQUORS</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>27031</t>
+          <t>74009</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>593 MAIN AVE</t>
+          <t>725 BROADWAY</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>PASSAIC</t>
+          <t>WESTWOOD</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
@@ -1849,12 +1849,12 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>KEYSTONE ICE</t>
+          <t>CAPE MAY BREWING COMPANY</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>CAPE MAY BREWING COMPANY</t>
         </is>
       </c>
       <c r="Q16" s="3" t="inlineStr">
@@ -1866,12 +1866,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>09/10/2026 11:46 AM</t>
+          <t>09/11/2026 08:55 AM</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1904,27 +1904,27 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>WINE GRAND (CARLSTADT)</t>
+          <t>HOME WINE LIQUOR (PASSAIC)</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>32017</t>
+          <t>27031</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>675 PATERSON AVE</t>
+          <t>593 MAIN AVE</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>CARLSTADT</t>
+          <t>PASSAIC</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>MBO</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
@@ -1951,22 +1951,22 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>09/09/2026 12:40 PM</t>
+          <t>09/10/2026 11:46 AM</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Jayson Romine</t>
+          <t>Matthew Powierski</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1985,26 +1985,26 @@
         </is>
       </c>
       <c r="H18" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB OF NEWTON (A)</t>
+          <t>WINE GRAND (CARLSTADT)</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>230412</t>
+          <t>32017</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>17 HAMPTON HOUSE ROAD</t>
+          <t>675 PATERSON AVE</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>NEWTON</t>
+          <t>CARLSTADT</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
@@ -2019,12 +2019,12 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>ATHLETIC BREWING CO</t>
+          <t>KEYSTONE ICE</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>ATHLETIC BREWING COMPANY</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q18" s="3" t="inlineStr">
@@ -2041,7 +2041,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -2070,7 +2070,7 @@
         </is>
       </c>
       <c r="H19" s="2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
@@ -2104,12 +2104,12 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>TALKHOUSE ENCORE VARIETY PACK</t>
+          <t>ATHLETIC BREWING CO</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>TALKHOUSE ENCORE</t>
+          <t>ATHLETIC BREWING COMPANY</t>
         </is>
       </c>
       <c r="Q19" s="3" t="inlineStr">
@@ -2126,7 +2126,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -2189,12 +2189,12 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISER ICED TEA + VODKA, CLASSIC ICED TEA</t>
+          <t>TALKHOUSE ENCORE VARIETY PACK</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>TALKHOUSE ENCORE</t>
         </is>
       </c>
       <c r="Q20" s="3" t="inlineStr">
@@ -2211,7 +2211,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -2274,7 +2274,7 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISER ICED TEA + VODKA, HALF &amp; HALF</t>
+          <t>SUN CRUISER ICED TEA + VODKA, CLASSIC ICED TEA</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
@@ -2296,7 +2296,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>8.3</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -2359,7 +2359,7 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISER ICED TEA VODKA VARIETY 18 PACK</t>
+          <t>SUN CRUISER ICED TEA + VODKA, HALF &amp; HALF</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>8.4</t>
+          <t>8.3</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -2444,7 +2444,7 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISERS RTD</t>
+          <t>SUN CRUISER ICED TEA VODKA VARIETY 18 PACK</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
@@ -2466,7 +2466,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>8.4</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -2495,7 +2495,7 @@
         </is>
       </c>
       <c r="H24" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
@@ -2529,12 +2529,12 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>SUN CRUISERS RTD</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q24" s="3" t="inlineStr">
@@ -2546,22 +2546,22 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>09/09/2026 10:37 AM</t>
+          <t>09/09/2026 12:40 PM</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Jayson Romine</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -2580,31 +2580,31 @@
         </is>
       </c>
       <c r="H25" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>WINELAND</t>
+          <t>USA WINE TRADERS CLUB OF NEWTON (A)</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>50020</t>
+          <t>230412</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>247 DEGRAW AVE</t>
+          <t>17 HAMPTON HOUSE ROAD</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>TEANECK</t>
+          <t>NEWTON</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>MBO</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
@@ -2614,10 +2614,14 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>MONACO</t>
-        </is>
-      </c>
-      <c r="P25" s="2" t="n"/>
+          <t>CAPE MAY BREWING COMPANY</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>CAPE MAY BREWING COMPANY</t>
+        </is>
+      </c>
       <c r="Q25" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
@@ -2627,22 +2631,22 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 12:28 PM</t>
+          <t>09/09/2026 10:37 AM</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Mike Ast</t>
+          <t>Chris Payton</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
+          <t>Michael Engel</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -2665,22 +2669,22 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>WALDWICK WINE/SPIRITS</t>
+          <t>WINELAND</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>88005</t>
+          <t>50020</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>23 WYCKOFF AVE</t>
+          <t>247 DEGRAW AVE</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>WALDWICK</t>
+          <t>TEANECK</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
@@ -2695,14 +2699,10 @@
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISERS RTD</t>
-        </is>
-      </c>
-      <c r="P26" s="2" t="inlineStr">
-        <is>
-          <t>BOSTON BEER COMPANY</t>
-        </is>
-      </c>
+          <t>MONACO</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="n"/>
       <c r="Q26" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
@@ -2717,7 +2717,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -2780,12 +2780,12 @@
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>BLUE MOON BELGIAN WHITE ALE</t>
+          <t>SUN CRUISERS RTD</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q27" s="3" t="inlineStr">
@@ -2797,22 +2797,22 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 12:17 PM</t>
+          <t>09/08/2026 12:28 PM</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Derrick laws</t>
+          <t>Mike Ast</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Denise Montes</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -2835,22 +2835,22 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>RAPHAEL &amp; ANGEL LIQ (A)</t>
+          <t>WALDWICK WINE/SPIRITS</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>20080</t>
+          <t>88005</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>390 MAIN ST</t>
+          <t>23 WYCKOFF AVE</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>PATERSON</t>
+          <t>WALDWICK</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
@@ -2865,7 +2865,7 @@
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>COORS LIGHT BEER</t>
+          <t>BLUE MOON BELGIAN WHITE ALE</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
@@ -2882,12 +2882,12 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 11:37 AM</t>
+          <t>09/08/2026 12:17 PM</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -2920,17 +2920,17 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>THE LIQUOR SHOP</t>
+          <t>RAPHAEL &amp; ANGEL LIQ (A)</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>21033</t>
+          <t>20080</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>498 E 30TH STREET</t>
+          <t>390 MAIN ST</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
@@ -2950,12 +2950,12 @@
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>MODELO CHELADA</t>
+          <t>COORS LIGHT BEER</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q29" s="3" t="inlineStr">
@@ -2967,12 +2967,12 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 11:35 AM</t>
+          <t>09/08/2026 11:37 AM</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -3035,12 +3035,12 @@
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>CERVEZA REPUBLICA LA TUYA 5.0 LA DURA</t>
+          <t>MODELO CHELADA</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>VINAIO IMPORTS LTD</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q30" s="3" t="inlineStr">
@@ -3052,12 +3052,12 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 11:34 AM</t>
+          <t>09/08/2026 11:35 AM</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -3120,12 +3120,12 @@
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>MODELO ORO</t>
+          <t>CERVEZA REPUBLICA LA TUYA 5.0 LA DURA</t>
         </is>
       </c>
       <c r="P31" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>VINAIO IMPORTS LTD</t>
         </is>
       </c>
       <c r="Q31" s="3" t="inlineStr">
@@ -3137,12 +3137,12 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 11:32 AM</t>
+          <t>09/08/2026 11:34 AM</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -3205,7 +3205,7 @@
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>MODELO ESPECIAL</t>
+          <t>MODELO ORO</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr">
@@ -3222,22 +3222,22 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:34 AM</t>
+          <t>09/08/2026 11:32 AM</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Derrick laws</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -3260,22 +3260,22 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
+          <t>THE LIQUOR SHOP</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>76010</t>
+          <t>21033</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>66 MARKET ST</t>
+          <t>498 E 30TH STREET</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>SADDLE BROOK</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
@@ -3290,12 +3290,12 @@
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>CARBLISS</t>
+          <t>MODELO ESPECIAL</t>
         </is>
       </c>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>DRINK CARBLISS</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q33" s="3" t="inlineStr">
@@ -3307,12 +3307,12 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:33 AM</t>
+          <t>09/03/2026 11:34 AM</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -3375,12 +3375,12 @@
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>TRULY HARD SELTZER</t>
+          <t>CARBLISS</t>
         </is>
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>DRINK CARBLISS</t>
         </is>
       </c>
       <c r="Q34" s="3" t="inlineStr">
@@ -3392,12 +3392,12 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:32 AM</t>
+          <t>09/03/2026 11:33 AM</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -3460,12 +3460,12 @@
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>COORS LIGHT BEER</t>
+          <t>TRULY HARD SELTZER</t>
         </is>
       </c>
       <c r="P35" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q35" s="3" t="inlineStr">
@@ -3477,12 +3477,12 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:31 AM</t>
+          <t>09/03/2026 11:32 AM</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -3545,12 +3545,12 @@
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>CORONA EXTRA</t>
+          <t>COORS LIGHT BEER</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q36" s="3" t="inlineStr">
@@ -3567,7 +3567,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -3630,7 +3630,7 @@
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>MODELO ESPECIAL</t>
+          <t>CORONA EXTRA</t>
         </is>
       </c>
       <c r="P37" s="2" t="inlineStr">
@@ -3647,12 +3647,12 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:30 AM</t>
+          <t>09/03/2026 11:31 AM</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -3715,12 +3715,12 @@
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>MODELO ESPECIAL</t>
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q38" s="3" t="inlineStr">
@@ -3732,12 +3732,12 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:29 AM</t>
+          <t>09/03/2026 11:30 AM</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -3800,12 +3800,12 @@
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISERS RTD</t>
+          <t>CAPE MAY BREWING COMPANY</t>
         </is>
       </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>CAPE MAY BREWING COMPANY</t>
         </is>
       </c>
       <c r="Q39" s="3" t="inlineStr">
@@ -3817,22 +3817,22 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:11 AM</t>
+          <t>09/03/2026 11:29 AM</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Mike Ast</t>
+          <t>Chris Payton</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
+          <t>Michael Engel</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -3855,22 +3855,22 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>FAIR LAWN WINE &amp; SPIRITS</t>
+          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>81006</t>
+          <t>76010</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>21-00 MAPLE AVE</t>
+          <t>66 MARKET ST</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>FAIR LAWN</t>
+          <t>SADDLE BROOK</t>
         </is>
       </c>
       <c r="M40" s="2" t="inlineStr">
@@ -3902,22 +3902,22 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 10:31 AM</t>
+          <t>09/03/2026 11:11 AM</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Mike Ast</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -3940,22 +3940,22 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON DISC LIQ (A)</t>
+          <t>FAIR LAWN WINE &amp; SPIRITS</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>25045</t>
+          <t>81006</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>73 ACKERMAN AVE BOTONY PL</t>
+          <t>21-00 MAPLE AVE</t>
         </is>
       </c>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON</t>
+          <t>FAIR LAWN</t>
         </is>
       </c>
       <c r="M41" s="2" t="inlineStr">
@@ -3970,12 +3970,12 @@
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>CARBLISS</t>
+          <t>SUN CRUISERS RTD</t>
         </is>
       </c>
       <c r="P41" s="2" t="inlineStr">
         <is>
-          <t>DRINK CARBLISS</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q41" s="3" t="inlineStr">
@@ -3987,12 +3987,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 10:30 AM</t>
+          <t>09/03/2026 10:31 AM</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -4055,12 +4055,12 @@
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>CORONA EXTRA</t>
+          <t>CARBLISS</t>
         </is>
       </c>
       <c r="P42" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>DRINK CARBLISS</t>
         </is>
       </c>
       <c r="Q42" s="3" t="inlineStr">
@@ -4072,12 +4072,12 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 10:29 AM</t>
+          <t>09/03/2026 10:30 AM</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -4140,7 +4140,7 @@
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>MODELO ESPECIAL</t>
+          <t>CORONA EXTRA</t>
         </is>
       </c>
       <c r="P43" s="2" t="inlineStr">
@@ -4157,12 +4157,12 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 10:28 AM</t>
+          <t>09/03/2026 10:29 AM</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -4225,12 +4225,12 @@
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>COORS LIGHT BEER</t>
+          <t>MODELO ESPECIAL</t>
         </is>
       </c>
       <c r="P44" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q44" s="3" t="inlineStr">
@@ -4247,7 +4247,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -4310,7 +4310,7 @@
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>MILLER LITE BEER</t>
+          <t>COORS LIGHT BEER</t>
         </is>
       </c>
       <c r="P45" s="2" t="inlineStr">
@@ -4327,83 +4327,168 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
+          <t>09/03/2026 10:28 AM</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>11.2</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Chris Payton</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Michael Engel</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON DISC LIQ (A)</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>25045</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>73 ACKERMAN AVE BOTONY PL</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>MBO</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="inlineStr">
+        <is>
+          <t>Cooler Door Wrap</t>
+        </is>
+      </c>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>MILLER LITE BEER</t>
+        </is>
+      </c>
+      <c r="P46" s="2" t="inlineStr">
+        <is>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
+        </is>
+      </c>
+      <c r="Q46" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
           <t>09/03/2026 10:27 AM</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>12.1</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>Chris Payton</t>
         </is>
       </c>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>Michael Engel</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>Ashley Furman</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="F47" s="2" t="inlineStr">
         <is>
           <t>Sales Rep</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="G47" s="2" t="inlineStr">
         <is>
           <t>Feature Activation</t>
         </is>
       </c>
-      <c r="H46" s="2" t="n">
+      <c r="H47" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="I46" s="2" t="inlineStr">
+      <c r="I47" s="2" t="inlineStr">
         <is>
           <t>CLIFTON DISC LIQ (A)</t>
         </is>
       </c>
-      <c r="J46" s="2" t="inlineStr">
+      <c r="J47" s="2" t="inlineStr">
         <is>
           <t>25045</t>
         </is>
       </c>
-      <c r="K46" s="2" t="inlineStr">
+      <c r="K47" s="2" t="inlineStr">
         <is>
           <t>73 ACKERMAN AVE BOTONY PL</t>
         </is>
       </c>
-      <c r="L46" s="2" t="inlineStr">
+      <c r="L47" s="2" t="inlineStr">
         <is>
           <t>CLIFTON</t>
         </is>
       </c>
-      <c r="M46" s="2" t="inlineStr">
+      <c r="M47" s="2" t="inlineStr">
         <is>
           <t>MBO</t>
         </is>
       </c>
-      <c r="N46" s="2" t="inlineStr">
+      <c r="N47" s="2" t="inlineStr">
         <is>
           <t>Cooler Door Wrap</t>
         </is>
       </c>
-      <c r="O46" s="2" t="inlineStr">
+      <c r="O47" s="2" t="inlineStr">
         <is>
           <t>MODELO CHELADA</t>
         </is>
       </c>
-      <c r="P46" s="2" t="inlineStr">
+      <c r="P47" s="2" t="inlineStr">
         <is>
           <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
-      <c r="Q46" s="3" t="inlineStr">
+      <c r="Q47" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
         </is>
@@ -4456,6 +4541,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q47" r:id="rId46"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Off-prem MPOs: 9/30 refresh -- W&S, Constellation, Promos_Report_39; Keystone and Corona synced
Wine & Spirits 360 -> 381 new placements (Brian Sengebush new at goal),
Constellation 1,270 -> 1,271 (Jayson Romine), one new cooler-door
sticker (Klejdi Lamo). Keystone and Fever Tree exports match the 9/29
pull. Sync rules applied: keystone-ice/actuals.csv and the incentive
tracker's Corona Gaintain file had stayed on the 9/28 pull; both caught
up and rebuilt (Keystone 202 -> 216 accounts, 8 -> 10 qualified). Hub
cache tag bumped for the new program_data.js.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MKEPYk6YSQsdW7mR8WAxwM
</commit_message>
<xml_diff>
--- a/MPOs/off-prem/pos_cooler_door_promos.xlsx
+++ b/MPOs/off-prem/pos_cooler_door_promos.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q100"/>
+  <dimension ref="A1:Q101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21.7109375" customWidth="1" style="6" min="1" max="1"/>
@@ -591,7 +591,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>09/29/2026 12:30 PM</t>
+          <t>09/30/2026 09:46 AM</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -601,12 +601,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>phil Ernst</t>
+          <t>Klejdi Lamo</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -629,27 +629,27 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>BOTTLE KING (A) GLEN ROCK</t>
+          <t>SAM'S LIQ WINE (P)</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>83010</t>
+          <t>190802</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>909 PROSPECT ST</t>
+          <t>325 W CLINTON ST</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>GLEN ROCK</t>
+          <t>DOVER</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Incentive</t>
+          <t>MBO</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -676,12 +676,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>09/28/2026 02:29 PM</t>
+          <t>09/29/2026 12:30 PM</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -714,22 +714,22 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>SUPER WINE WAREHSE(P)PATE</t>
+          <t>BOTTLE KING (A) GLEN ROCK</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>20106</t>
+          <t>83010</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>42 E 30TH ST</t>
+          <t>909 PROSPECT ST</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>PATERSON</t>
+          <t>GLEN ROCK</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -761,12 +761,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>09/28/2026 12:25 PM</t>
+          <t>09/28/2026 02:29 PM</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -799,22 +799,22 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>CITY SUPERMARKET</t>
+          <t>SUPER WINE WAREHSE(P)PATE</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>43001</t>
+          <t>20106</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>289 BERGEN BLVD</t>
+          <t>42 E 30TH ST</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>FAIRVIEW</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -846,22 +846,22 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>09/28/2026 12:16 PM</t>
+          <t>09/28/2026 12:25 PM</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>patrick infante</t>
+          <t>phil Ernst</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Denise Montes</t>
+          <t>Michael Engel</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -871,7 +871,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -884,22 +884,22 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>SHOPPERS VINEYARD (A)</t>
+          <t>CITY SUPERMARKET</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>24011</t>
+          <t>43001</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>875 BLOOMFIELD AVE</t>
+          <t>289 BERGEN BLVD</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON</t>
+          <t>FAIRVIEW</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -914,12 +914,12 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>MODELO ESPECIAL</t>
+          <t>KEYSTONE ICE</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q5" s="3" t="inlineStr">
@@ -931,22 +931,22 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>09/28/2026 11:43 AM</t>
+          <t>09/28/2026 12:16 PM</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Daniel La Gala</t>
+          <t>patrick infante</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -956,7 +956,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -969,27 +969,27 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>BUY RITE OF FAIRVIEW</t>
+          <t>SHOPPERS VINEYARD (A)</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>43013</t>
+          <t>24011</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>201 BROAD AVE</t>
+          <t>875 BLOOMFIELD AVE</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>FAIRVIEW</t>
+          <t>CLIFTON</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>MBO</t>
+          <t>Incentive</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -999,7 +999,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>CORONA EXTRA</t>
+          <t>MODELO ESPECIAL</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1016,17 +1016,17 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>09/28/2026 11:03 AM</t>
+          <t>09/28/2026 11:43 AM</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Dave Ehlers</t>
+          <t>Daniel La Gala</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -1054,27 +1054,27 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>DELI MART (A)</t>
+          <t>BUY RITE OF FAIRVIEW</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>41012</t>
+          <t>43013</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>789 MAIN ST</t>
+          <t>201 BROAD AVE</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>HACKENSACK</t>
+          <t>FAIRVIEW</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>MBO</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1084,12 +1084,12 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>KEYSTONE ICE</t>
+          <t>CORONA EXTRA</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q7" s="3" t="inlineStr">
@@ -1101,22 +1101,22 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>09/28/2026 10:59 AM</t>
+          <t>09/28/2026 11:03 AM</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Matthew Powierski</t>
+          <t>Dave Ehlers</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Denise Montes</t>
+          <t>Michael Engel</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1139,27 +1139,27 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>LUIGI'S LIQUOR (A)</t>
+          <t>DELI MART (A)</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>26001</t>
+          <t>41012</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>175 JEFFERSON ST</t>
+          <t>789 MAIN ST</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>PASSAIC</t>
+          <t>HACKENSACK</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>MBO</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1186,22 +1186,22 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>09/28/2026 10:48 AM</t>
+          <t>09/28/2026 10:59 AM</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Dave Ehlers</t>
+          <t>Matthew Powierski</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1224,27 +1224,27 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>GEORGE'S LIQ</t>
+          <t>LUIGI'S LIQUOR (A)</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>41005</t>
+          <t>26001</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>130 ANDERSON ST</t>
+          <t>175 JEFFERSON ST</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>HACKENSACK</t>
+          <t>PASSAIC</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>MBO</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1254,12 +1254,12 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>CORONA EXTRA</t>
+          <t>KEYSTONE ICE</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q9" s="3" t="inlineStr">
@@ -1271,12 +1271,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>09/28/2026 10:40 AM</t>
+          <t>09/28/2026 10:48 AM</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1339,12 +1339,12 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>FAMOSA LAGER</t>
+          <t>CORONA EXTRA</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>CENTRAL BEER IMPORT &amp; EXPORT FAMOSA</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q10" s="3" t="inlineStr">
@@ -1356,12 +1356,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>09/28/2026 10:38 AM</t>
+          <t>09/28/2026 10:40 AM</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1424,12 +1424,12 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>KEYSTONE ICE</t>
+          <t>FAMOSA LAGER</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>CENTRAL BEER IMPORT &amp; EXPORT FAMOSA</t>
         </is>
       </c>
       <c r="Q11" s="3" t="inlineStr">
@@ -1441,17 +1441,17 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>09/28/2026 10:25 AM</t>
+          <t>09/28/2026 10:38 AM</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>phil Ernst</t>
+          <t>Dave Ehlers</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1479,27 +1479,27 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>STEW LEONARD'S WINES &amp; SPIRITS OF CLIFTON</t>
+          <t>GEORGE'S LIQ</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>25010</t>
+          <t>41005</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>467 ALLWOOD RD</t>
+          <t>130 ANDERSON ST</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON</t>
+          <t>HACKENSACK</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>Incentive</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1526,17 +1526,17 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>09/28/2026 09:40 AM</t>
+          <t>09/28/2026 10:25 AM</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Dave Ehlers</t>
+          <t>phil Ernst</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1564,27 +1564,27 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>WINE AND LIQ DEPOT(A)</t>
+          <t>STEW LEONARD'S WINES &amp; SPIRITS OF CLIFTON</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>39012</t>
+          <t>25010</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>310 HUYLER ST</t>
+          <t>467 ALLWOOD RD</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>SOUTH HACKENSAC</t>
+          <t>CLIFTON</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Incentive</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
@@ -1594,10 +1594,14 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>MONACO</t>
-        </is>
-      </c>
-      <c r="P13" s="2" t="n"/>
+          <t>KEYSTONE ICE</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
+        </is>
+      </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
@@ -1607,12 +1611,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>09/28/2026 09:36 AM</t>
+          <t>09/28/2026 09:40 AM</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1675,14 +1679,10 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>KEYSTONE ICE</t>
-        </is>
-      </c>
-      <c r="P14" s="2" t="inlineStr">
-        <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
-        </is>
-      </c>
+          <t>MONACO</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="n"/>
       <c r="Q14" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
@@ -1692,22 +1692,22 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>09/23/2026 03:15 PM</t>
+          <t>09/28/2026 09:36 AM</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Pablo Lopez</t>
+          <t>Dave Ehlers</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Denise Montes</t>
+          <t>Michael Engel</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1730,27 +1730,27 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>COSTAMBAR BAR &amp; LIQUOR CORP.</t>
+          <t>WINE AND LIQ DEPOT(A)</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>20051</t>
+          <t>39012</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>292-294 MARKET STREET</t>
+          <t>310 HUYLER ST</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>PATERSON</t>
+          <t>SOUTH HACKENSAC</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>MBO, Incentive</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
@@ -1777,22 +1777,22 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>09/23/2026 02:43 PM</t>
+          <t>09/23/2026 03:15 PM</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>phil Ernst</t>
+          <t>Pablo Lopez</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1811,21 +1811,21 @@
         </is>
       </c>
       <c r="H16" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>SUPER WINE WAREHSE(P)PATE</t>
+          <t>COSTAMBAR BAR &amp; LIQUOR CORP.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>20106</t>
+          <t>20051</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>42 E 30TH ST</t>
+          <t>292-294 MARKET STREET</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>Incentive</t>
+          <t>MBO, Incentive</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>PERONI NASTRO AZZURRO</t>
+          <t>KEYSTONE ICE</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
@@ -1862,12 +1862,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>09/23/2026 02:42 PM</t>
+          <t>09/23/2026 02:43 PM</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1896,7 +1896,7 @@
         </is>
       </c>
       <c r="H17" s="2" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
@@ -1930,12 +1930,12 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>MODELO ESPECIAL</t>
+          <t>PERONI NASTRO AZZURRO</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q17" s="3" t="inlineStr">
@@ -1947,12 +1947,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>09/23/2026 02:39 PM</t>
+          <t>09/23/2026 02:42 PM</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1981,7 +1981,7 @@
         </is>
       </c>
       <c r="H18" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
@@ -2015,12 +2015,12 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>BLUE MOON BELGIAN WHITE ALE</t>
+          <t>MODELO ESPECIAL</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q18" s="3" t="inlineStr">
@@ -2032,12 +2032,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>09/23/2026 01:20 PM</t>
+          <t>09/23/2026 02:39 PM</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -2066,26 +2066,26 @@
         </is>
       </c>
       <c r="H19" s="2" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>FOOD UNIVERSE MARKETPLACE</t>
+          <t>SUPER WINE WAREHSE(P)PATE</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>83001</t>
+          <t>20106</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>937 LINCOLN AVE</t>
+          <t>42 E 30TH ST</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>GLEN ROCK</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
@@ -2100,10 +2100,14 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>MONACO</t>
-        </is>
-      </c>
-      <c r="P19" s="2" t="n"/>
+          <t>BLUE MOON BELGIAN WHITE ALE</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
+        </is>
+      </c>
       <c r="Q19" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
@@ -2113,12 +2117,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>09/23/2026 12:49 PM</t>
+          <t>09/23/2026 01:20 PM</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -2147,26 +2151,26 @@
         </is>
       </c>
       <c r="H20" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>SHOP RITE LIQ(A) FAIR LWN</t>
+          <t>FOOD UNIVERSE MARKETPLACE</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>81014</t>
+          <t>83001</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>35-07 BROADWAY</t>
+          <t>937 LINCOLN AVE</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>FAIR LAWN</t>
+          <t>GLEN ROCK</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
@@ -2181,14 +2185,10 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>TWISTED TEA ORIGINAL</t>
-        </is>
-      </c>
-      <c r="P20" s="2" t="inlineStr">
-        <is>
-          <t>BOSTON BEER COMPANY</t>
-        </is>
-      </c>
+          <t>MONACO</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="n"/>
       <c r="Q20" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
@@ -2198,12 +2198,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>09/23/2026 12:15 PM</t>
+          <t>09/23/2026 12:49 PM</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -2232,26 +2232,26 @@
         </is>
       </c>
       <c r="H21" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>SHOP RITE LIQ (PARAMUS)</t>
+          <t>SHOP RITE LIQ(A) FAIR LWN</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>80005</t>
+          <t>81014</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>224 RT 4 E</t>
+          <t>35-07 BROADWAY</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>PARAMUS</t>
+          <t>FAIR LAWN</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
@@ -2266,12 +2266,12 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>ARNOLD PALMER SPIKED</t>
+          <t>TWISTED TEA ORIGINAL</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q21" s="3" t="inlineStr">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>7.2</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -2317,7 +2317,7 @@
         </is>
       </c>
       <c r="H22" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
@@ -2351,7 +2351,7 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>SIMPLY SPIKED LEMONADE</t>
+          <t>ARNOLD PALMER SPIKED</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>7.3</t>
+          <t>7.2</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -2402,7 +2402,7 @@
         </is>
       </c>
       <c r="H23" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
@@ -2436,12 +2436,12 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>TWISTED TEA ORIGINAL</t>
+          <t>SIMPLY SPIKED LEMONADE</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q23" s="3" t="inlineStr">
@@ -2453,12 +2453,12 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>09/23/2026 12:14 PM</t>
+          <t>09/23/2026 12:15 PM</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>7.3</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -2487,7 +2487,7 @@
         </is>
       </c>
       <c r="H24" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>TRULY HARD SELTZER</t>
+          <t>TWISTED TEA ORIGINAL</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
@@ -2538,12 +2538,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>09/23/2026 12:12 PM</t>
+          <t>09/23/2026 12:14 PM</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -2572,7 +2572,7 @@
         </is>
       </c>
       <c r="H25" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
@@ -2606,12 +2606,12 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY IPA</t>
+          <t>TRULY HARD SELTZER</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q25" s="3" t="inlineStr">
@@ -2623,12 +2623,12 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>09/23/2026 12:10 PM</t>
+          <t>09/23/2026 12:12 PM</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -2657,7 +2657,7 @@
         </is>
       </c>
       <c r="H26" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
@@ -2691,12 +2691,12 @@
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>PERONI NASTRO AZZURRO</t>
+          <t>CAPE MAY IPA</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>CAPE MAY BREWING COMPANY</t>
         </is>
       </c>
       <c r="Q26" s="3" t="inlineStr">
@@ -2708,12 +2708,12 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>09/23/2026 12:09 PM</t>
+          <t>09/23/2026 12:10 PM</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -2742,7 +2742,7 @@
         </is>
       </c>
       <c r="H27" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
@@ -2776,12 +2776,12 @@
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>TRULY HARD SELTZER</t>
+          <t>PERONI NASTRO AZZURRO</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q27" s="3" t="inlineStr">
@@ -2793,12 +2793,12 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>09/23/2026 12:07 PM</t>
+          <t>09/23/2026 12:09 PM</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -2827,7 +2827,7 @@
         </is>
       </c>
       <c r="H28" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
@@ -2861,7 +2861,7 @@
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>TWISTED TEA ORIGINAL</t>
+          <t>TRULY HARD SELTZER</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
@@ -2878,12 +2878,12 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>09/23/2026 10:52 AM</t>
+          <t>09/23/2026 12:07 PM</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>13.1</t>
+          <t>12.1</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -2912,21 +2912,21 @@
         </is>
       </c>
       <c r="H29" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>PRIME WINE CELLAR LIQUOR &amp; BEER</t>
+          <t>SHOP RITE LIQ (PARAMUS)</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>80041</t>
+          <t>80005</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>396 RT 17 NORTH</t>
+          <t>224 RT 4 E</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
@@ -2946,10 +2946,14 @@
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>MONACO</t>
-        </is>
-      </c>
-      <c r="P29" s="2" t="n"/>
+          <t>TWISTED TEA ORIGINAL</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>BOSTON BEER COMPANY</t>
+        </is>
+      </c>
       <c r="Q29" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
@@ -2959,22 +2963,22 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>09/22/2026 02:09 PM</t>
+          <t>09/23/2026 10:52 AM</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>13.1</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Pablo Lopez</t>
+          <t>phil Ernst</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Denise Montes</t>
+          <t>Michael Engel</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -2997,27 +3001,27 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>SCHULMAN'S (P) DELI</t>
+          <t>PRIME WINE CELLAR LIQUOR &amp; BEER</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>21034</t>
+          <t>80041</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>521 PARK AVE</t>
+          <t>396 RT 17 NORTH</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>PATERSON</t>
+          <t>PARAMUS</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>MBO, Incentive</t>
+          <t>Incentive</t>
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr">
@@ -3027,14 +3031,10 @@
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>KEYSTONE ICE</t>
-        </is>
-      </c>
-      <c r="P30" s="2" t="inlineStr">
-        <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
-        </is>
-      </c>
+          <t>MONACO</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="n"/>
       <c r="Q30" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
@@ -3044,12 +3044,12 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>09/22/2026 01:37 PM</t>
+          <t>09/22/2026 02:09 PM</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -3082,17 +3082,17 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>CARABALLO'S</t>
+          <t>SCHULMAN'S (P) DELI</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>20022</t>
+          <t>21034</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>495 MARKET STREET</t>
+          <t>521 PARK AVE</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
@@ -3102,7 +3102,7 @@
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>Incentive, MBO</t>
+          <t>MBO, Incentive</t>
         </is>
       </c>
       <c r="N31" s="2" t="inlineStr">
@@ -3129,12 +3129,12 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>09/22/2026 01:01 PM</t>
+          <t>09/22/2026 01:37 PM</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -3167,17 +3167,17 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>ALTIERO LIQUORS</t>
+          <t>CARABALLO'S</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>21024</t>
+          <t>20022</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>498 ELLISON ST.</t>
+          <t>495 MARKET STREET</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
@@ -3187,7 +3187,7 @@
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>MBO, Incentive</t>
+          <t>Incentive, MBO</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr">
@@ -3214,22 +3214,22 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>09/22/2026 12:52 PM</t>
+          <t>09/22/2026 01:01 PM</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Daniel La Gala</t>
+          <t>Pablo Lopez</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -3252,27 +3252,27 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>BOULEVARD LIQ.(FAIRVIEW)</t>
+          <t>ALTIERO LIQUORS</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>43004</t>
+          <t>21024</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>153 BERGEN BLVD</t>
+          <t>498 ELLISON ST.</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>FAIRVIEW</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>MBO</t>
+          <t>MBO, Incentive</t>
         </is>
       </c>
       <c r="N33" s="2" t="inlineStr">
@@ -3282,12 +3282,12 @@
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>MODELO ESPECIAL</t>
+          <t>KEYSTONE ICE</t>
         </is>
       </c>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q33" s="3" t="inlineStr">
@@ -3299,22 +3299,22 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>09/22/2026 12:35 PM</t>
+          <t>09/22/2026 12:52 PM</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Pablo Lopez</t>
+          <t>Daniel La Gala</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Denise Montes</t>
+          <t>Michael Engel</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -3337,27 +3337,27 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>RIVERSIDE LIQUORS (PATERSON)</t>
+          <t>BOULEVARD LIQ.(FAIRVIEW)</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>20032</t>
+          <t>43004</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>402 RIVER ST</t>
+          <t>153 BERGEN BLVD</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>PATERSON</t>
+          <t>FAIRVIEW</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>MBO, Incentive</t>
+          <t>MBO</t>
         </is>
       </c>
       <c r="N34" s="2" t="inlineStr">
@@ -3367,12 +3367,12 @@
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>KEYSTONE ICE</t>
+          <t>MODELO ESPECIAL</t>
         </is>
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q34" s="3" t="inlineStr">
@@ -3384,12 +3384,12 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>09/22/2026 12:17 PM</t>
+          <t>09/22/2026 12:35 PM</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -3422,17 +3422,17 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>GENE'S LIQUOR</t>
+          <t>RIVERSIDE LIQUORS (PATERSON)</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>15016</t>
+          <t>20032</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>26 N STRAIGHT ST</t>
+          <t>402 RIVER ST</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
@@ -3469,17 +3469,17 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>09/22/2026 12:15 PM</t>
+          <t>09/22/2026 12:17 PM</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>James Heaney</t>
+          <t>Pablo Lopez</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -3507,27 +3507,27 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>LUCKY 7 (A)</t>
+          <t>GENE'S LIQUOR</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>28012</t>
+          <t>15016</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>77 RIVER RD</t>
+          <t>26 N STRAIGHT ST</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>NORTH ARLINGTON</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>MBO</t>
+          <t>MBO, Incentive</t>
         </is>
       </c>
       <c r="N36" s="2" t="inlineStr">
@@ -3537,12 +3537,12 @@
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>TWISTED TEA ORIGINAL</t>
+          <t>KEYSTONE ICE</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q36" s="3" t="inlineStr">
@@ -3554,12 +3554,12 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>09/22/2026 12:14 PM</t>
+          <t>09/22/2026 12:15 PM</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -3622,12 +3622,12 @@
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>KEYSTONE ICE</t>
+          <t>TWISTED TEA ORIGINAL</t>
         </is>
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q37" s="3" t="inlineStr">
@@ -3639,12 +3639,12 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>09/22/2026 11:45 AM</t>
+          <t>09/22/2026 12:14 PM</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -3673,21 +3673,21 @@
         </is>
       </c>
       <c r="H38" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>METRO LIQUORS (NORTH ARLINGTON)</t>
+          <t>LUCKY 7 (A)</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>28007</t>
+          <t>28012</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>17 SCHUYLER AVE</t>
+          <t>77 RIVER RD</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
@@ -3707,12 +3707,12 @@
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISERS RTD</t>
+          <t>KEYSTONE ICE</t>
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q38" s="3" t="inlineStr">
@@ -3724,17 +3724,17 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>09/22/2026 11:29 AM</t>
+          <t>09/22/2026 11:45 AM</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Pablo Lopez</t>
+          <t>James Heaney</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -3758,31 +3758,31 @@
         </is>
       </c>
       <c r="H39" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>JOE'S LIQUOR (A)</t>
+          <t>METRO LIQUORS (NORTH ARLINGTON)</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>20070</t>
+          <t>28007</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>328 11TH AVE</t>
+          <t>17 SCHUYLER AVE</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>PATERSON</t>
+          <t>NORTH ARLINGTON</t>
         </is>
       </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>MBO, Incentive</t>
+          <t>MBO</t>
         </is>
       </c>
       <c r="N39" s="2" t="inlineStr">
@@ -3792,12 +3792,12 @@
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>KEYSTONE ICE</t>
+          <t>SUN CRUISERS RTD</t>
         </is>
       </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q39" s="3" t="inlineStr">
@@ -3809,17 +3809,17 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>09/22/2026 11:07 AM</t>
+          <t>09/22/2026 11:29 AM</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>James Heaney</t>
+          <t>Pablo Lopez</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -3847,27 +3847,27 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>LIQUOR SHED</t>
+          <t>JOE'S LIQUOR (A)</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>29003</t>
+          <t>20070</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>740 RIDGE ROAD</t>
+          <t>328 11TH AVE</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>LYNDHURST</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M40" s="2" t="inlineStr">
         <is>
-          <t>MBO</t>
+          <t>MBO, Incentive</t>
         </is>
       </c>
       <c r="N40" s="2" t="inlineStr">
@@ -3877,12 +3877,12 @@
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>TWISTED TEA ORIGINAL</t>
+          <t>KEYSTONE ICE</t>
         </is>
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q40" s="3" t="inlineStr">
@@ -3894,22 +3894,22 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>09/22/2026 11:04 AM</t>
+          <t>09/22/2026 11:07 AM</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Daniel La Gala</t>
+          <t>James Heaney</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -3932,22 +3932,22 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>METRO LIQUOR (CLIFFSIDE PARK)</t>
+          <t>LIQUOR SHED</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>44009</t>
+          <t>29003</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>341 GORGE RD.</t>
+          <t>740 RIDGE ROAD</t>
         </is>
       </c>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>CLIFFSIDE PARK</t>
+          <t>LYNDHURST</t>
         </is>
       </c>
       <c r="M41" s="2" t="inlineStr">
@@ -3962,10 +3962,14 @@
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>MONACO</t>
-        </is>
-      </c>
-      <c r="P41" s="2" t="n"/>
+          <t>TWISTED TEA ORIGINAL</t>
+        </is>
+      </c>
+      <c r="P41" s="2" t="inlineStr">
+        <is>
+          <t>BOSTON BEER COMPANY</t>
+        </is>
+      </c>
       <c r="Q41" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
@@ -3975,22 +3979,22 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>09/22/2026 10:53 AM</t>
+          <t>09/22/2026 11:04 AM</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>13.1</t>
+          <t>12.1</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Pablo Lopez</t>
+          <t>Daniel La Gala</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Denise Montes</t>
+          <t>Michael Engel</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -4013,27 +4017,27 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>BOMBOLON LIQUOR &amp; GROCERY</t>
+          <t>METRO LIQUOR (CLIFFSIDE PARK)</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>20014</t>
+          <t>44009</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>192 E 16TH ST</t>
+          <t>341 GORGE RD.</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>PATERSON</t>
+          <t>CLIFFSIDE PARK</t>
         </is>
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>Incentive, MBO</t>
+          <t>MBO</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
@@ -4043,14 +4047,10 @@
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>KEYSTONE ICE</t>
-        </is>
-      </c>
-      <c r="P42" s="2" t="inlineStr">
-        <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
-        </is>
-      </c>
+          <t>MONACO</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="n"/>
       <c r="Q42" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
@@ -4060,22 +4060,22 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>09/22/2026 10:42 AM</t>
+          <t>09/22/2026 10:53 AM</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>14.1</t>
+          <t>13.1</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Daniel La Gala</t>
+          <t>Pablo Lopez</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -4098,27 +4098,27 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>WINE AND FOOD MART (Z)</t>
+          <t>BOMBOLON LIQUOR &amp; GROCERY</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>44002</t>
+          <t>20014</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>589 ANDERSON AVE</t>
+          <t>192 E 16TH ST</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>CLIFFSIDE PARK</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M43" s="2" t="inlineStr">
         <is>
-          <t>MBO</t>
+          <t>Incentive, MBO</t>
         </is>
       </c>
       <c r="N43" s="2" t="inlineStr">
@@ -4128,7 +4128,7 @@
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>COORS LIGHT BEER</t>
+          <t>KEYSTONE ICE</t>
         </is>
       </c>
       <c r="P43" s="2" t="inlineStr">
@@ -4150,7 +4150,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>15.1</t>
+          <t>14.1</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -4213,12 +4213,12 @@
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>HEINEKEN</t>
+          <t>COORS LIGHT BEER</t>
         </is>
       </c>
       <c r="P44" s="2" t="inlineStr">
         <is>
-          <t>HEINEKEN</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q44" s="3" t="inlineStr">
@@ -4230,22 +4230,22 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>09/21/2026 02:54 PM</t>
+          <t>09/22/2026 10:42 AM</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>16.1</t>
+          <t>15.1</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Pablo Lopez</t>
+          <t>Daniel La Gala</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Denise Montes</t>
+          <t>Michael Engel</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -4268,27 +4268,27 @@
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>#1 LIQRS (P)</t>
+          <t>WINE AND FOOD MART (Z)</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>27005</t>
+          <t>44002</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>130 HOWE AVE</t>
+          <t>589 ANDERSON AVE</t>
         </is>
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>PASSAIC</t>
+          <t>CLIFFSIDE PARK</t>
         </is>
       </c>
       <c r="M45" s="2" t="inlineStr">
         <is>
-          <t>MBO, Incentive</t>
+          <t>MBO</t>
         </is>
       </c>
       <c r="N45" s="2" t="inlineStr">
@@ -4298,12 +4298,12 @@
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>KEYSTONE ICE</t>
+          <t>HEINEKEN</t>
         </is>
       </c>
       <c r="P45" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>HEINEKEN</t>
         </is>
       </c>
       <c r="Q45" s="3" t="inlineStr">
@@ -4315,12 +4315,12 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>09/21/2026 02:34 PM</t>
+          <t>09/21/2026 02:54 PM</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>17.1</t>
+          <t>16.1</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -4353,17 +4353,17 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>JOHNNY'S LIQS (P)</t>
+          <t>#1 LIQRS (P)</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>27021</t>
+          <t>27005</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>370 MONROE ST</t>
+          <t>130 HOWE AVE</t>
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr">
@@ -4400,12 +4400,12 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>09/21/2026 01:56 PM</t>
+          <t>09/21/2026 02:34 PM</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>18.1</t>
+          <t>17.1</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -4438,17 +4438,17 @@
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>MONROE WINE &amp; LIQ(P)</t>
+          <t>JOHNNY'S LIQS (P)</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>27043</t>
+          <t>27021</t>
         </is>
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>199 MONROE ST</t>
+          <t>370 MONROE ST</t>
         </is>
       </c>
       <c r="L47" s="2" t="inlineStr">
@@ -4458,7 +4458,7 @@
       </c>
       <c r="M47" s="2" t="inlineStr">
         <is>
-          <t>Incentive, MBO</t>
+          <t>MBO, Incentive</t>
         </is>
       </c>
       <c r="N47" s="2" t="inlineStr">
@@ -4485,12 +4485,12 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>09/21/2026 01:46 PM</t>
+          <t>09/21/2026 01:56 PM</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>19.1</t>
+          <t>18.1</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -4523,17 +4523,17 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>BROADWAY W&amp;L</t>
+          <t>MONROE WINE &amp; LIQ(P)</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>27069</t>
+          <t>27043</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>62 BROADWAY</t>
+          <t>199 MONROE ST</t>
         </is>
       </c>
       <c r="L48" s="2" t="inlineStr">
@@ -4570,12 +4570,12 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>09/21/2026 01:23 PM</t>
+          <t>09/21/2026 01:46 PM</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>20.1</t>
+          <t>19.1</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -4608,17 +4608,17 @@
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>SUNNY'S LIQS.(P)</t>
+          <t>BROADWAY W&amp;L</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>27066</t>
+          <t>27069</t>
         </is>
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>413 MONROE ST</t>
+          <t>62 BROADWAY</t>
         </is>
       </c>
       <c r="L49" s="2" t="inlineStr">
@@ -4655,12 +4655,12 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>09/21/2026 12:58 PM</t>
+          <t>09/21/2026 01:23 PM</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>21.1</t>
+          <t>20.1</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -4693,17 +4693,17 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>REGALADO LIQ</t>
+          <t>SUNNY'S LIQS.(P)</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>26014</t>
+          <t>27066</t>
         </is>
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>168 MARKET ST</t>
+          <t>413 MONROE ST</t>
         </is>
       </c>
       <c r="L50" s="2" t="inlineStr">
@@ -4740,12 +4740,12 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>09/21/2026 12:38 PM</t>
+          <t>09/21/2026 12:58 PM</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>22.1</t>
+          <t>21.1</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -4778,17 +4778,17 @@
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>PASSAIC DISCOUNT LIQUORS</t>
+          <t>REGALADO LIQ</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>27072</t>
+          <t>26014</t>
         </is>
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>49 MARKET ST</t>
+          <t>168 MARKET ST</t>
         </is>
       </c>
       <c r="L51" s="2" t="inlineStr">
@@ -4798,7 +4798,7 @@
       </c>
       <c r="M51" s="2" t="inlineStr">
         <is>
-          <t>MBO, Incentive</t>
+          <t>Incentive, MBO</t>
         </is>
       </c>
       <c r="N51" s="2" t="inlineStr">
@@ -4825,22 +4825,22 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>09/21/2026 10:54 AM</t>
+          <t>09/21/2026 12:38 PM</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>23.1</t>
+          <t>22.1</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Jayson Romine</t>
+          <t>Pablo Lopez</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -4859,31 +4859,31 @@
         </is>
       </c>
       <c r="H52" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>PATRICKS WINE BARN</t>
+          <t>PASSAIC DISCOUNT LIQUORS</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>231316</t>
+          <t>27072</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>38 HAMBURG AVE</t>
+          <t>49 MARKET ST</t>
         </is>
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>SUSSEX</t>
+          <t>PASSAIC</t>
         </is>
       </c>
       <c r="M52" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>MBO, Incentive</t>
         </is>
       </c>
       <c r="N52" s="2" t="inlineStr">
@@ -4893,7 +4893,7 @@
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>ARNOLD PALMER SPIKED HALF &amp; HALF</t>
+          <t>KEYSTONE ICE</t>
         </is>
       </c>
       <c r="P52" s="2" t="inlineStr">
@@ -4910,22 +4910,22 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>09/21/2026 10:45 AM</t>
+          <t>09/21/2026 10:54 AM</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>24.1</t>
+          <t>23.1</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Matthew Powierski</t>
+          <t>Jayson Romine</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Denise Montes</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -4944,31 +4944,31 @@
         </is>
       </c>
       <c r="H53" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>KING LIQUORS</t>
+          <t>PATRICKS WINE BARN</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>36016</t>
+          <t>231316</t>
         </is>
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>434 MAIN AVE</t>
+          <t>38 HAMBURG AVE</t>
         </is>
       </c>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>WALLINGTON</t>
+          <t>SUSSEX</t>
         </is>
       </c>
       <c r="M53" s="2" t="inlineStr">
         <is>
-          <t>MBO</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N53" s="2" t="inlineStr">
@@ -4978,7 +4978,7 @@
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>KEYSTONE ICE</t>
+          <t>ARNOLD PALMER SPIKED HALF &amp; HALF</t>
         </is>
       </c>
       <c r="P53" s="2" t="inlineStr">
@@ -4995,17 +4995,17 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>09/21/2026 10:32 AM</t>
+          <t>09/21/2026 10:45 AM</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>25.1</t>
+          <t>24.1</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Pablo Lopez</t>
+          <t>Matthew Powierski</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -5033,27 +5033,27 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>LEGACY BAR &amp; LIQUOR</t>
+          <t>KING LIQUORS</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>15040</t>
+          <t>36016</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>1019 MCBRIDE AVE</t>
+          <t>434 MAIN AVE</t>
         </is>
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>WOODLAND PARK</t>
+          <t>WALLINGTON</t>
         </is>
       </c>
       <c r="M54" s="2" t="inlineStr">
         <is>
-          <t>MBO, Incentive</t>
+          <t>MBO</t>
         </is>
       </c>
       <c r="N54" s="2" t="inlineStr">
@@ -5080,12 +5080,12 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>09/17/2026 12:44 PM</t>
+          <t>09/21/2026 10:32 AM</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>25.1</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -5118,27 +5118,27 @@
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>INTENSITY LOUNGE/ANGIE'S LIQUORS</t>
+          <t>LEGACY BAR &amp; LIQUOR</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>20062</t>
+          <t>15040</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>109 MAIN ST</t>
+          <t>1019 MCBRIDE AVE</t>
         </is>
       </c>
       <c r="L55" s="2" t="inlineStr">
         <is>
-          <t>PATERSON</t>
+          <t>WOODLAND PARK</t>
         </is>
       </c>
       <c r="M55" s="2" t="inlineStr">
         <is>
-          <t>Incentive</t>
+          <t>MBO, Incentive</t>
         </is>
       </c>
       <c r="N55" s="2" t="inlineStr">
@@ -5165,7 +5165,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 01:16 PM</t>
+          <t>09/17/2026 12:44 PM</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -5175,7 +5175,7 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Matthew Powierski</t>
+          <t>Pablo Lopez</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -5203,27 +5203,27 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>METRO LIQUORS (EAST RUTHERFORD)</t>
+          <t>INTENSITY LOUNGE/ANGIE'S LIQUORS</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>31004</t>
+          <t>20062</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>576 PATERSON AVE</t>
+          <t>109 MAIN ST</t>
         </is>
       </c>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>EAST RUTHERFORD</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M56" s="2" t="inlineStr">
         <is>
-          <t>MBO</t>
+          <t>Incentive</t>
         </is>
       </c>
       <c r="N56" s="2" t="inlineStr">
@@ -5250,7 +5250,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>09/15/2026 12:07 PM</t>
+          <t>09/16/2026 01:16 PM</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -5260,12 +5260,12 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Mike Ast</t>
+          <t>Matthew Powierski</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -5288,22 +5288,22 @@
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>WALDWICK WINE/SPIRITS</t>
+          <t>METRO LIQUORS (EAST RUTHERFORD)</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>88005</t>
+          <t>31004</t>
         </is>
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>23 WYCKOFF AVE</t>
+          <t>576 PATERSON AVE</t>
         </is>
       </c>
       <c r="L57" s="2" t="inlineStr">
         <is>
-          <t>WALDWICK</t>
+          <t>EAST RUTHERFORD</t>
         </is>
       </c>
       <c r="M57" s="2" t="inlineStr">
@@ -5318,12 +5318,12 @@
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>POP SIPS GINGER LIME</t>
+          <t>KEYSTONE ICE</t>
         </is>
       </c>
       <c r="P57" s="2" t="inlineStr">
         <is>
-          <t>PASSION TREE</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q57" s="3" t="inlineStr">
@@ -5340,7 +5340,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -5403,7 +5403,7 @@
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>POP SIPS RASPBERRY ROSE</t>
+          <t>POP SIPS GINGER LIME</t>
         </is>
       </c>
       <c r="P58" s="2" t="inlineStr">
@@ -5425,7 +5425,7 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -5488,7 +5488,7 @@
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>POP SIPS VARIETY 8PK</t>
+          <t>POP SIPS RASPBERRY ROSE</t>
         </is>
       </c>
       <c r="P59" s="2" t="inlineStr">
@@ -5505,12 +5505,12 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>09/15/2026 12:05 PM</t>
+          <t>09/15/2026 12:07 PM</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -5573,12 +5573,12 @@
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>COORS LIGHT BEER</t>
+          <t>POP SIPS VARIETY 8PK</t>
         </is>
       </c>
       <c r="P60" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>PASSION TREE</t>
         </is>
       </c>
       <c r="Q60" s="3" t="inlineStr">
@@ -5595,7 +5595,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -5658,7 +5658,7 @@
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>MILLER LITE BEER</t>
+          <t>COORS LIGHT BEER</t>
         </is>
       </c>
       <c r="P61" s="2" t="inlineStr">
@@ -5675,17 +5675,17 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>09/14/2026 09:50 AM</t>
+          <t>09/15/2026 12:05 PM</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>2.2</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Shane Barreca</t>
+          <t>Mike Ast</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -5709,26 +5709,26 @@
         </is>
       </c>
       <c r="H62" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>SHOP RITE LIQ (A)HILLSDAL</t>
+          <t>WALDWICK WINE/SPIRITS</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>73008</t>
+          <t>88005</t>
         </is>
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>371 BROADWAY</t>
+          <t>23 WYCKOFF AVE</t>
         </is>
       </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>HILLSDALE</t>
+          <t>WALDWICK</t>
         </is>
       </c>
       <c r="M62" s="2" t="inlineStr">
@@ -5743,12 +5743,12 @@
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>TWISTED TEA ORIGINAL</t>
+          <t>MILLER LITE BEER</t>
         </is>
       </c>
       <c r="P62" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q62" s="3" t="inlineStr">
@@ -5760,7 +5760,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>09/14/2026 07:38 AM</t>
+          <t>09/14/2026 09:50 AM</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -5794,26 +5794,26 @@
         </is>
       </c>
       <c r="H63" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>WINEMART DISCOUNT</t>
+          <t>SHOP RITE LIQ (A)HILLSDAL</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>74005</t>
+          <t>73008</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>700 BROADWAY SUITE 42</t>
+          <t>371 BROADWAY</t>
         </is>
       </c>
       <c r="L63" s="2" t="inlineStr">
         <is>
-          <t>WESTWOOD</t>
+          <t>HILLSDALE</t>
         </is>
       </c>
       <c r="M63" s="2" t="inlineStr">
@@ -5828,12 +5828,12 @@
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>NIGHT SHIFT X CAPE MAY BREWBERRY</t>
+          <t>TWISTED TEA ORIGINAL</t>
         </is>
       </c>
       <c r="P63" s="2" t="inlineStr">
         <is>
-          <t>NIGHT SHIFT BREWING</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q63" s="3" t="inlineStr">
@@ -5845,12 +5845,12 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>09/14/2026 07:36 AM</t>
+          <t>09/14/2026 07:38 AM</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -5883,17 +5883,17 @@
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>WESTWOOD WINE AND LIQUORS</t>
+          <t>WINEMART DISCOUNT</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>74009</t>
+          <t>74005</t>
         </is>
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>725 BROADWAY</t>
+          <t>700 BROADWAY SUITE 42</t>
         </is>
       </c>
       <c r="L64" s="2" t="inlineStr">
@@ -5913,12 +5913,12 @@
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>ATHLETIC BREWING CO</t>
+          <t>NIGHT SHIFT X CAPE MAY BREWBERRY</t>
         </is>
       </c>
       <c r="P64" s="2" t="inlineStr">
         <is>
-          <t>ATHLETIC BREWING COMPANY</t>
+          <t>NIGHT SHIFT BREWING</t>
         </is>
       </c>
       <c r="Q64" s="3" t="inlineStr">
@@ -5930,12 +5930,12 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>09/14/2026 07:35 AM</t>
+          <t>09/14/2026 07:36 AM</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -5968,22 +5968,22 @@
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>GARDEN STATE DELI (A)</t>
+          <t>WESTWOOD WINE AND LIQUORS</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>62001</t>
+          <t>74009</t>
         </is>
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>135 OAKLAND AVE</t>
+          <t>725 BROADWAY</t>
         </is>
       </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>CLOSTER</t>
+          <t>WESTWOOD</t>
         </is>
       </c>
       <c r="M65" s="2" t="inlineStr">
@@ -5998,12 +5998,12 @@
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>CORONA EXTRA</t>
+          <t>ATHLETIC BREWING CO</t>
         </is>
       </c>
       <c r="P65" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>ATHLETIC BREWING COMPANY</t>
         </is>
       </c>
       <c r="Q65" s="3" t="inlineStr">
@@ -6020,7 +6020,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>CORONA LIGHT</t>
+          <t>CORONA EXTRA</t>
         </is>
       </c>
       <c r="P66" s="2" t="inlineStr">
@@ -6105,7 +6105,7 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -6168,7 +6168,7 @@
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>CORONA PREMIER</t>
+          <t>CORONA LIGHT</t>
         </is>
       </c>
       <c r="P67" s="2" t="inlineStr">
@@ -6190,7 +6190,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>3.3</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -6253,7 +6253,7 @@
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>MODELO ESPECIAL</t>
+          <t>CORONA PREMIER</t>
         </is>
       </c>
       <c r="P68" s="2" t="inlineStr">
@@ -6270,12 +6270,12 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>09/14/2026 07:31 AM</t>
+          <t>09/14/2026 07:35 AM</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>3.4</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -6308,22 +6308,22 @@
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>WESTWOOD WINE AND LIQUORS</t>
+          <t>GARDEN STATE DELI (A)</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>74009</t>
+          <t>62001</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
-          <t>725 BROADWAY</t>
+          <t>135 OAKLAND AVE</t>
         </is>
       </c>
       <c r="L69" s="2" t="inlineStr">
         <is>
-          <t>WESTWOOD</t>
+          <t>CLOSTER</t>
         </is>
       </c>
       <c r="M69" s="2" t="inlineStr">
@@ -6338,12 +6338,12 @@
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>MODELO ESPECIAL</t>
         </is>
       </c>
       <c r="P69" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q69" s="3" t="inlineStr">
@@ -6355,22 +6355,22 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>09/11/2026 08:55 AM</t>
+          <t>09/14/2026 07:31 AM</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Matthew Powierski</t>
+          <t>Shane Barreca</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Denise Montes</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -6393,22 +6393,22 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>HOME WINE LIQUOR (PASSAIC)</t>
+          <t>WESTWOOD WINE AND LIQUORS</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>27031</t>
+          <t>74009</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr">
         <is>
-          <t>593 MAIN AVE</t>
+          <t>725 BROADWAY</t>
         </is>
       </c>
       <c r="L70" s="2" t="inlineStr">
         <is>
-          <t>PASSAIC</t>
+          <t>WESTWOOD</t>
         </is>
       </c>
       <c r="M70" s="2" t="inlineStr">
@@ -6423,12 +6423,12 @@
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>KEYSTONE ICE</t>
+          <t>CAPE MAY BREWING COMPANY</t>
         </is>
       </c>
       <c r="P70" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>CAPE MAY BREWING COMPANY</t>
         </is>
       </c>
       <c r="Q70" s="3" t="inlineStr">
@@ -6440,12 +6440,12 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>09/10/2026 11:46 AM</t>
+          <t>09/11/2026 08:55 AM</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -6478,27 +6478,27 @@
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>WINE GRAND (CARLSTADT)</t>
+          <t>HOME WINE LIQUOR (PASSAIC)</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>32017</t>
+          <t>27031</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr">
         <is>
-          <t>675 PATERSON AVE</t>
+          <t>593 MAIN AVE</t>
         </is>
       </c>
       <c r="L71" s="2" t="inlineStr">
         <is>
-          <t>CARLSTADT</t>
+          <t>PASSAIC</t>
         </is>
       </c>
       <c r="M71" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>MBO</t>
         </is>
       </c>
       <c r="N71" s="2" t="inlineStr">
@@ -6525,22 +6525,22 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>09/09/2026 12:40 PM</t>
+          <t>09/10/2026 11:46 AM</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Jayson Romine</t>
+          <t>Matthew Powierski</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -6559,26 +6559,26 @@
         </is>
       </c>
       <c r="H72" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB OF NEWTON (A)</t>
+          <t>WINE GRAND (CARLSTADT)</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>230412</t>
+          <t>32017</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>17 HAMPTON HOUSE ROAD</t>
+          <t>675 PATERSON AVE</t>
         </is>
       </c>
       <c r="L72" s="2" t="inlineStr">
         <is>
-          <t>NEWTON</t>
+          <t>CARLSTADT</t>
         </is>
       </c>
       <c r="M72" s="2" t="inlineStr">
@@ -6593,12 +6593,12 @@
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>ATHLETIC BREWING CO</t>
+          <t>KEYSTONE ICE</t>
         </is>
       </c>
       <c r="P72" s="2" t="inlineStr">
         <is>
-          <t>ATHLETIC BREWING COMPANY</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q72" s="3" t="inlineStr">
@@ -6615,7 +6615,7 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
@@ -6644,7 +6644,7 @@
         </is>
       </c>
       <c r="H73" s="2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
@@ -6678,12 +6678,12 @@
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>TALKHOUSE ENCORE VARIETY PACK</t>
+          <t>ATHLETIC BREWING CO</t>
         </is>
       </c>
       <c r="P73" s="2" t="inlineStr">
         <is>
-          <t>TALKHOUSE ENCORE</t>
+          <t>ATHLETIC BREWING COMPANY</t>
         </is>
       </c>
       <c r="Q73" s="3" t="inlineStr">
@@ -6700,7 +6700,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -6763,12 +6763,12 @@
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISER ICED TEA + VODKA, CLASSIC ICED TEA</t>
+          <t>TALKHOUSE ENCORE VARIETY PACK</t>
         </is>
       </c>
       <c r="P74" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>TALKHOUSE ENCORE</t>
         </is>
       </c>
       <c r="Q74" s="3" t="inlineStr">
@@ -6785,7 +6785,7 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -6848,7 +6848,7 @@
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISER ICED TEA + VODKA, HALF &amp; HALF</t>
+          <t>SUN CRUISER ICED TEA + VODKA, CLASSIC ICED TEA</t>
         </is>
       </c>
       <c r="P75" s="2" t="inlineStr">
@@ -6870,7 +6870,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>8.3</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -6933,7 +6933,7 @@
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISER ICED TEA VODKA VARIETY 18 PACK</t>
+          <t>SUN CRUISER ICED TEA + VODKA, HALF &amp; HALF</t>
         </is>
       </c>
       <c r="P76" s="2" t="inlineStr">
@@ -6955,7 +6955,7 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>8.4</t>
+          <t>8.3</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
@@ -7018,7 +7018,7 @@
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISERS RTD</t>
+          <t>SUN CRUISER ICED TEA VODKA VARIETY 18 PACK</t>
         </is>
       </c>
       <c r="P77" s="2" t="inlineStr">
@@ -7040,7 +7040,7 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>8.4</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -7069,7 +7069,7 @@
         </is>
       </c>
       <c r="H78" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
@@ -7103,12 +7103,12 @@
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>SUN CRUISERS RTD</t>
         </is>
       </c>
       <c r="P78" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q78" s="3" t="inlineStr">
@@ -7120,22 +7120,22 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>09/09/2026 10:37 AM</t>
+          <t>09/09/2026 12:40 PM</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Jayson Romine</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
@@ -7154,31 +7154,31 @@
         </is>
       </c>
       <c r="H79" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t>WINELAND</t>
+          <t>USA WINE TRADERS CLUB OF NEWTON (A)</t>
         </is>
       </c>
       <c r="J79" s="2" t="inlineStr">
         <is>
-          <t>50020</t>
+          <t>230412</t>
         </is>
       </c>
       <c r="K79" s="2" t="inlineStr">
         <is>
-          <t>247 DEGRAW AVE</t>
+          <t>17 HAMPTON HOUSE ROAD</t>
         </is>
       </c>
       <c r="L79" s="2" t="inlineStr">
         <is>
-          <t>TEANECK</t>
+          <t>NEWTON</t>
         </is>
       </c>
       <c r="M79" s="2" t="inlineStr">
         <is>
-          <t>MBO</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N79" s="2" t="inlineStr">
@@ -7188,10 +7188,14 @@
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>MONACO</t>
-        </is>
-      </c>
-      <c r="P79" s="2" t="n"/>
+          <t>CAPE MAY BREWING COMPANY</t>
+        </is>
+      </c>
+      <c r="P79" s="2" t="inlineStr">
+        <is>
+          <t>CAPE MAY BREWING COMPANY</t>
+        </is>
+      </c>
       <c r="Q79" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
@@ -7201,22 +7205,22 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 12:28 PM</t>
+          <t>09/09/2026 10:37 AM</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Mike Ast</t>
+          <t>Chris Payton</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
+          <t>Michael Engel</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -7239,22 +7243,22 @@
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>WALDWICK WINE/SPIRITS</t>
+          <t>WINELAND</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
         <is>
-          <t>88005</t>
+          <t>50020</t>
         </is>
       </c>
       <c r="K80" s="2" t="inlineStr">
         <is>
-          <t>23 WYCKOFF AVE</t>
+          <t>247 DEGRAW AVE</t>
         </is>
       </c>
       <c r="L80" s="2" t="inlineStr">
         <is>
-          <t>WALDWICK</t>
+          <t>TEANECK</t>
         </is>
       </c>
       <c r="M80" s="2" t="inlineStr">
@@ -7269,14 +7273,10 @@
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISERS RTD</t>
-        </is>
-      </c>
-      <c r="P80" s="2" t="inlineStr">
-        <is>
-          <t>BOSTON BEER COMPANY</t>
-        </is>
-      </c>
+          <t>MONACO</t>
+        </is>
+      </c>
+      <c r="P80" s="2" t="n"/>
       <c r="Q80" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
@@ -7291,7 +7291,7 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
@@ -7354,12 +7354,12 @@
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>BLUE MOON BELGIAN WHITE ALE</t>
+          <t>SUN CRUISERS RTD</t>
         </is>
       </c>
       <c r="P81" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q81" s="3" t="inlineStr">
@@ -7371,22 +7371,22 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 12:17 PM</t>
+          <t>09/08/2026 12:28 PM</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Derrick laws</t>
+          <t>Mike Ast</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Denise Montes</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
@@ -7409,22 +7409,22 @@
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>RAPHAEL &amp; ANGEL LIQ (A)</t>
+          <t>WALDWICK WINE/SPIRITS</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
         <is>
-          <t>20080</t>
+          <t>88005</t>
         </is>
       </c>
       <c r="K82" s="2" t="inlineStr">
         <is>
-          <t>390 MAIN ST</t>
+          <t>23 WYCKOFF AVE</t>
         </is>
       </c>
       <c r="L82" s="2" t="inlineStr">
         <is>
-          <t>PATERSON</t>
+          <t>WALDWICK</t>
         </is>
       </c>
       <c r="M82" s="2" t="inlineStr">
@@ -7439,7 +7439,7 @@
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>COORS LIGHT BEER</t>
+          <t>BLUE MOON BELGIAN WHITE ALE</t>
         </is>
       </c>
       <c r="P82" s="2" t="inlineStr">
@@ -7456,12 +7456,12 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 11:37 AM</t>
+          <t>09/08/2026 12:17 PM</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
@@ -7494,17 +7494,17 @@
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>THE LIQUOR SHOP</t>
+          <t>RAPHAEL &amp; ANGEL LIQ (A)</t>
         </is>
       </c>
       <c r="J83" s="2" t="inlineStr">
         <is>
-          <t>21033</t>
+          <t>20080</t>
         </is>
       </c>
       <c r="K83" s="2" t="inlineStr">
         <is>
-          <t>498 E 30TH STREET</t>
+          <t>390 MAIN ST</t>
         </is>
       </c>
       <c r="L83" s="2" t="inlineStr">
@@ -7524,12 +7524,12 @@
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>MODELO CHELADA</t>
+          <t>COORS LIGHT BEER</t>
         </is>
       </c>
       <c r="P83" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q83" s="3" t="inlineStr">
@@ -7541,12 +7541,12 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 11:35 AM</t>
+          <t>09/08/2026 11:37 AM</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -7609,12 +7609,12 @@
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>CERVEZA REPUBLICA LA TUYA 5.0 LA DURA</t>
+          <t>MODELO CHELADA</t>
         </is>
       </c>
       <c r="P84" s="2" t="inlineStr">
         <is>
-          <t>VINAIO IMPORTS LTD</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q84" s="3" t="inlineStr">
@@ -7626,12 +7626,12 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 11:34 AM</t>
+          <t>09/08/2026 11:35 AM</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
@@ -7694,12 +7694,12 @@
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>MODELO ORO</t>
+          <t>CERVEZA REPUBLICA LA TUYA 5.0 LA DURA</t>
         </is>
       </c>
       <c r="P85" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>VINAIO IMPORTS LTD</t>
         </is>
       </c>
       <c r="Q85" s="3" t="inlineStr">
@@ -7711,12 +7711,12 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 11:32 AM</t>
+          <t>09/08/2026 11:34 AM</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
@@ -7779,7 +7779,7 @@
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>MODELO ESPECIAL</t>
+          <t>MODELO ORO</t>
         </is>
       </c>
       <c r="P86" s="2" t="inlineStr">
@@ -7796,22 +7796,22 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:34 AM</t>
+          <t>09/08/2026 11:32 AM</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Derrick laws</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
@@ -7834,22 +7834,22 @@
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
+          <t>THE LIQUOR SHOP</t>
         </is>
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>76010</t>
+          <t>21033</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr">
         <is>
-          <t>66 MARKET ST</t>
+          <t>498 E 30TH STREET</t>
         </is>
       </c>
       <c r="L87" s="2" t="inlineStr">
         <is>
-          <t>SADDLE BROOK</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M87" s="2" t="inlineStr">
@@ -7864,12 +7864,12 @@
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>CARBLISS</t>
+          <t>MODELO ESPECIAL</t>
         </is>
       </c>
       <c r="P87" s="2" t="inlineStr">
         <is>
-          <t>DRINK CARBLISS</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q87" s="3" t="inlineStr">
@@ -7881,12 +7881,12 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:33 AM</t>
+          <t>09/03/2026 11:34 AM</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
@@ -7949,12 +7949,12 @@
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>TRULY HARD SELTZER</t>
+          <t>CARBLISS</t>
         </is>
       </c>
       <c r="P88" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>DRINK CARBLISS</t>
         </is>
       </c>
       <c r="Q88" s="3" t="inlineStr">
@@ -7966,12 +7966,12 @@
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:32 AM</t>
+          <t>09/03/2026 11:33 AM</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
@@ -8034,12 +8034,12 @@
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>COORS LIGHT BEER</t>
+          <t>TRULY HARD SELTZER</t>
         </is>
       </c>
       <c r="P89" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q89" s="3" t="inlineStr">
@@ -8051,12 +8051,12 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:31 AM</t>
+          <t>09/03/2026 11:32 AM</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
@@ -8119,12 +8119,12 @@
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>CORONA EXTRA</t>
+          <t>COORS LIGHT BEER</t>
         </is>
       </c>
       <c r="P90" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q90" s="3" t="inlineStr">
@@ -8141,7 +8141,7 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
@@ -8204,7 +8204,7 @@
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>MODELO ESPECIAL</t>
+          <t>CORONA EXTRA</t>
         </is>
       </c>
       <c r="P91" s="2" t="inlineStr">
@@ -8221,12 +8221,12 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:30 AM</t>
+          <t>09/03/2026 11:31 AM</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
@@ -8289,12 +8289,12 @@
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>MODELO ESPECIAL</t>
         </is>
       </c>
       <c r="P92" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q92" s="3" t="inlineStr">
@@ -8306,12 +8306,12 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:29 AM</t>
+          <t>09/03/2026 11:30 AM</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
@@ -8374,12 +8374,12 @@
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISERS RTD</t>
+          <t>CAPE MAY BREWING COMPANY</t>
         </is>
       </c>
       <c r="P93" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>CAPE MAY BREWING COMPANY</t>
         </is>
       </c>
       <c r="Q93" s="3" t="inlineStr">
@@ -8391,22 +8391,22 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:11 AM</t>
+          <t>09/03/2026 11:29 AM</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Mike Ast</t>
+          <t>Chris Payton</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
+          <t>Michael Engel</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -8429,22 +8429,22 @@
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>FAIR LAWN WINE &amp; SPIRITS</t>
+          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
         <is>
-          <t>81006</t>
+          <t>76010</t>
         </is>
       </c>
       <c r="K94" s="2" t="inlineStr">
         <is>
-          <t>21-00 MAPLE AVE</t>
+          <t>66 MARKET ST</t>
         </is>
       </c>
       <c r="L94" s="2" t="inlineStr">
         <is>
-          <t>FAIR LAWN</t>
+          <t>SADDLE BROOK</t>
         </is>
       </c>
       <c r="M94" s="2" t="inlineStr">
@@ -8476,22 +8476,22 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 10:31 AM</t>
+          <t>09/03/2026 11:11 AM</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Mike Ast</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
@@ -8514,22 +8514,22 @@
       </c>
       <c r="I95" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON DISC LIQ (A)</t>
+          <t>FAIR LAWN WINE &amp; SPIRITS</t>
         </is>
       </c>
       <c r="J95" s="2" t="inlineStr">
         <is>
-          <t>25045</t>
+          <t>81006</t>
         </is>
       </c>
       <c r="K95" s="2" t="inlineStr">
         <is>
-          <t>73 ACKERMAN AVE BOTONY PL</t>
+          <t>21-00 MAPLE AVE</t>
         </is>
       </c>
       <c r="L95" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON</t>
+          <t>FAIR LAWN</t>
         </is>
       </c>
       <c r="M95" s="2" t="inlineStr">
@@ -8544,12 +8544,12 @@
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>CARBLISS</t>
+          <t>SUN CRUISERS RTD</t>
         </is>
       </c>
       <c r="P95" s="2" t="inlineStr">
         <is>
-          <t>DRINK CARBLISS</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q95" s="3" t="inlineStr">
@@ -8561,12 +8561,12 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 10:30 AM</t>
+          <t>09/03/2026 10:31 AM</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
@@ -8629,12 +8629,12 @@
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>CORONA EXTRA</t>
+          <t>CARBLISS</t>
         </is>
       </c>
       <c r="P96" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>DRINK CARBLISS</t>
         </is>
       </c>
       <c r="Q96" s="3" t="inlineStr">
@@ -8646,12 +8646,12 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 10:29 AM</t>
+          <t>09/03/2026 10:30 AM</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
@@ -8714,7 +8714,7 @@
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>MODELO ESPECIAL</t>
+          <t>CORONA EXTRA</t>
         </is>
       </c>
       <c r="P97" s="2" t="inlineStr">
@@ -8731,12 +8731,12 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 10:28 AM</t>
+          <t>09/03/2026 10:29 AM</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
@@ -8799,12 +8799,12 @@
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>COORS LIGHT BEER</t>
+          <t>MODELO ESPECIAL</t>
         </is>
       </c>
       <c r="P98" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q98" s="3" t="inlineStr">
@@ -8821,7 +8821,7 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>11.1</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
@@ -8884,7 +8884,7 @@
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>MILLER LITE BEER</t>
+          <t>COORS LIGHT BEER</t>
         </is>
       </c>
       <c r="P99" s="2" t="inlineStr">
@@ -8901,83 +8901,168 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
+          <t>09/03/2026 10:28 AM</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>11.2</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>Chris Payton</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>Michael Engel</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I100" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON DISC LIQ (A)</t>
+        </is>
+      </c>
+      <c r="J100" s="2" t="inlineStr">
+        <is>
+          <t>25045</t>
+        </is>
+      </c>
+      <c r="K100" s="2" t="inlineStr">
+        <is>
+          <t>73 ACKERMAN AVE BOTONY PL</t>
+        </is>
+      </c>
+      <c r="L100" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON</t>
+        </is>
+      </c>
+      <c r="M100" s="2" t="inlineStr">
+        <is>
+          <t>MBO</t>
+        </is>
+      </c>
+      <c r="N100" s="2" t="inlineStr">
+        <is>
+          <t>Cooler Door Wrap</t>
+        </is>
+      </c>
+      <c r="O100" s="2" t="inlineStr">
+        <is>
+          <t>MILLER LITE BEER</t>
+        </is>
+      </c>
+      <c r="P100" s="2" t="inlineStr">
+        <is>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
+        </is>
+      </c>
+      <c r="Q100" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
           <t>09/03/2026 10:27 AM</t>
         </is>
       </c>
-      <c r="B100" s="2" t="inlineStr">
+      <c r="B101" s="2" t="inlineStr">
         <is>
           <t>12.1</t>
         </is>
       </c>
-      <c r="C100" s="2" t="inlineStr">
+      <c r="C101" s="2" t="inlineStr">
         <is>
           <t>Chris Payton</t>
         </is>
       </c>
-      <c r="D100" s="2" t="inlineStr">
+      <c r="D101" s="2" t="inlineStr">
         <is>
           <t>Michael Engel</t>
         </is>
       </c>
-      <c r="E100" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
-      <c r="F100" s="2" t="inlineStr">
-        <is>
-          <t>Sales Rep</t>
-        </is>
-      </c>
-      <c r="G100" s="2" t="inlineStr">
-        <is>
-          <t>Feature Activation</t>
-        </is>
-      </c>
-      <c r="H100" s="2" t="n">
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="I100" s="2" t="inlineStr">
+      <c r="I101" s="2" t="inlineStr">
         <is>
           <t>CLIFTON DISC LIQ (A)</t>
         </is>
       </c>
-      <c r="J100" s="2" t="inlineStr">
+      <c r="J101" s="2" t="inlineStr">
         <is>
           <t>25045</t>
         </is>
       </c>
-      <c r="K100" s="2" t="inlineStr">
+      <c r="K101" s="2" t="inlineStr">
         <is>
           <t>73 ACKERMAN AVE BOTONY PL</t>
         </is>
       </c>
-      <c r="L100" s="2" t="inlineStr">
+      <c r="L101" s="2" t="inlineStr">
         <is>
           <t>CLIFTON</t>
         </is>
       </c>
-      <c r="M100" s="2" t="inlineStr">
+      <c r="M101" s="2" t="inlineStr">
         <is>
           <t>MBO</t>
         </is>
       </c>
-      <c r="N100" s="2" t="inlineStr">
-        <is>
-          <t>Cooler Door Wrap</t>
-        </is>
-      </c>
-      <c r="O100" s="2" t="inlineStr">
+      <c r="N101" s="2" t="inlineStr">
+        <is>
+          <t>Cooler Door Wrap</t>
+        </is>
+      </c>
+      <c r="O101" s="2" t="inlineStr">
         <is>
           <t>MODELO CHELADA</t>
         </is>
       </c>
-      <c r="P100" s="2" t="inlineStr">
+      <c r="P101" s="2" t="inlineStr">
         <is>
           <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
-      <c r="Q100" s="3" t="inlineStr">
+      <c r="Q101" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
         </is>
@@ -9084,6 +9169,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q98" r:id="rId97"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q99" r:id="rId98"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q100" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q101" r:id="rId100"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>